<commit_message>
upgrade: update snapshot 20260401; add support U,DAI;
</commit_message>
<xml_diff>
--- a/snapshot/huobi_por.xlsx
+++ b/snapshot/huobi_por.xlsx
@@ -4,12 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15200"/>
+    <workbookView windowWidth="27860" windowHeight="15680"/>
   </bookViews>
   <sheets>
     <sheet name="huobi_por" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0" calcOnSave="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="138">
   <si>
     <t>coin</t>
   </si>
@@ -62,19 +62,19 @@
     <t>DOGE</t>
   </si>
   <si>
-    <t>ETH(ALL)</t>
+    <t>ETH(All)</t>
   </si>
   <si>
     <t>ETH</t>
   </si>
   <si>
-    <t>aETH</t>
+    <t>Morpho-ETH</t>
   </si>
   <si>
     <t>stETH</t>
   </si>
   <si>
-    <t>HTX(ALL)</t>
+    <t>HTX(All)</t>
   </si>
   <si>
     <t>HTX-ERC20</t>
@@ -89,7 +89,7 @@
     <t>SOL</t>
   </si>
   <si>
-    <t>TRX(ALL)</t>
+    <t>TRX(All)</t>
   </si>
   <si>
     <t>TRX</t>
@@ -104,16 +104,19 @@
     <t>ERC20-USDC</t>
   </si>
   <si>
-    <t>STEAK-USDC</t>
-  </si>
-  <si>
-    <t>BEP20-USDC</t>
-  </si>
-  <si>
-    <t>BASE-USDC</t>
-  </si>
-  <si>
-    <t>USDT(ALL)</t>
+    <t>spUSDC-ERC20</t>
+  </si>
+  <si>
+    <t>U(All)</t>
+  </si>
+  <si>
+    <t>BEP20-U</t>
+  </si>
+  <si>
+    <t>STEAK-U</t>
+  </si>
+  <si>
+    <t>USDT(All)</t>
   </si>
   <si>
     <t>stUSDT-TRC20</t>
@@ -131,15 +134,12 @@
     <t>jUSDT-TRC20</t>
   </si>
   <si>
+    <t>spUSDT-ERC20</t>
+  </si>
+  <si>
     <t>USDT-aEthUSDT</t>
   </si>
   <si>
-    <t>USDT-BEP20</t>
-  </si>
-  <si>
-    <t>USDT-Morpho</t>
-  </si>
-  <si>
     <t>WLFI(All)</t>
   </si>
   <si>
@@ -152,6 +152,12 @@
     <t>XRP</t>
   </si>
   <si>
+    <t>DAI(All)</t>
+  </si>
+  <si>
+    <t>ERC20-DAI</t>
+  </si>
+  <si>
     <t>address</t>
   </si>
   <si>
@@ -326,12 +332,6 @@
     <t>8NBEbxLknGv5aRYefFrW2qFXoDZyi9fSHJNiJRvEcMBE</t>
   </si>
   <si>
-    <t>0xafdfd157d9361e621e476036fee62f688450692b</t>
-  </si>
-  <si>
-    <t>0xd5eb44e88c27f972d96f58677c7ebcf581102286</t>
-  </si>
-  <si>
     <t>0xa77ff0e1c52f58363a53282624c7baa5fa91687d</t>
   </si>
   <si>
@@ -362,12 +362,6 @@
     <t>0x3ca7a1fcc5306107b4bd37c82359ec2a1c62b32658bb01201f12bf5e9e1b5c54623f440d226165bf4d216cffe5a4e3fce9e636e7514eac5c29af97df12e88fd400</t>
   </si>
   <si>
-    <t>TBuzWQynfzershAsPfGjo4A9sXUfZf8wsq</t>
-  </si>
-  <si>
-    <t>851fc5515cd6b0f94f28939de7d4f6977740aa60dc81754b64c2f110e6f1db1e1465e0d1fe3885a0f5b3fb3b4a807b4ba06c84a1a79ae91d7bea62b1ef47300001</t>
-  </si>
-  <si>
     <t>rKUDvXFJMFu65LqPTH3Yfpii4rbKT9bSQT</t>
   </si>
   <si>
@@ -377,10 +371,10 @@
     <t>rneMKXXdKMD1R9WZ4Yqv1bfst6bjpaD5tP</t>
   </si>
   <si>
-    <t>DL2EGukahtib57Sg7FtHsvf8HgwMJtbBA3</t>
-  </si>
-  <si>
-    <t>DQhEuTa5UkNcD8YFZK3pvjFfrtMqQpJhSa</t>
+    <t>DJX3kCZfcDuREturnUNKEBQELi1PFaLkJC</t>
+  </si>
+  <si>
+    <t>DLzCvKskasu4Adj3XgbyNitKBukBSa5JPP</t>
   </si>
   <si>
     <t>DRRU8L7fF4k9w7SF3Z6ei8onPCsh9hjGX1</t>
@@ -404,9 +398,6 @@
     <t>DJxVuu8KDh7qKfuieJoWQNFYmK1L3k773X</t>
   </si>
   <si>
-    <t>ACELftry9PkuRkWr86njdGUC3xbbkZyhfc</t>
-  </si>
-  <si>
     <t>DQkukxxY7LYdb2bchK8Zgo14wwyEPsHVJf</t>
   </si>
   <si>
@@ -419,22 +410,37 @@
     <t>DB5KWytcxHyphHPn9iC92Y9JqPRL1Fq21p</t>
   </si>
   <si>
-    <t>9x25QJUvtejNqQATCUz4WkdQK32MGcKaQA</t>
-  </si>
-  <si>
-    <t>A8rDxpAb592psxQyttVSE1jwcUrreVFuRx</t>
-  </si>
-  <si>
-    <t>A56RUMzWPSTfqU1oygE7oYgNaRD4KD25CL</t>
-  </si>
-  <si>
-    <t>9roa2rnj4JdJ3WPv69rwsR5fTqKdro7ARZ</t>
-  </si>
-  <si>
-    <t>A8Z3ba7JEwPetjkM9uhpu2LBm5ToyU5sNL</t>
-  </si>
-  <si>
-    <t>A1NkCSL992iBmx9bvKhTf17nZjf4fDxaBs</t>
+    <t>9uucMrtiGcTY2bMSt7A3VVYBCPk2kzGogb</t>
+  </si>
+  <si>
+    <t>A4925JsPyQyQiYubyn5zQ4KC9y6iJkS1e1</t>
+  </si>
+  <si>
+    <t>9yU8uyXdwS5zZuyjFHUfqGs18GaMfSNzUs</t>
+  </si>
+  <si>
+    <t>A43g9V6kwrExQjHyso5MgukHCLCcUdGQ3H</t>
+  </si>
+  <si>
+    <t>9t53SAmQPL1svuUiMFWuEqugvrLSCWDjxS</t>
+  </si>
+  <si>
+    <t>A4yEfPjBCJDtRBV6kPrf4ueiJEvHYpWhvA</t>
+  </si>
+  <si>
+    <t>9vba9CCV84vFoiSaiYViiF35JGUSDsfAdt</t>
+  </si>
+  <si>
+    <t>9x564hoR6kESz9Q6zhscrh5VEgau53ZbFv</t>
+  </si>
+  <si>
+    <t>ABjCPgbwfDi4QBcsYDx7sSjcTkW7cdbZMz</t>
+  </si>
+  <si>
+    <t>AAthcUZK8pb2s6Sb3rTWiN3iJHgBWAraar</t>
+  </si>
+  <si>
+    <t>AFVYXnSSB2eiPLXLsRv1pFnUMM7HFXgLXA</t>
   </si>
 </sst>
 </file>
@@ -449,7 +455,7 @@
     <numFmt numFmtId="176" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="177" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -489,25 +495,26 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线 Light"/>
-      <charset val="134"/>
-      <scheme val="major"/>
-    </font>
-    <font>
       <i/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF7F7F7F"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -535,77 +542,84 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color theme="0"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF9C5700"/>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="0"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -803,7 +817,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -845,7 +859,7 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thick">
+      <bottom style="medium">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -854,17 +868,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thick">
+      <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.399975585192419"/>
       </bottom>
       <diagonal/>
     </border>
@@ -959,7 +964,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -974,31 +979,31 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1013,77 +1018,77 @@
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1098,6 +1103,9 @@
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
@@ -1444,7 +1452,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="17.6" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="23.1666666666667" customWidth="1"/>
@@ -1474,7 +1482,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="3">
-        <v>21362.98</v>
+        <v>21524.14</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1482,10 +1490,10 @@
         <v>5</v>
       </c>
       <c r="B3" s="2">
-        <v>938735</v>
+        <v>943083</v>
       </c>
       <c r="C3" s="3">
-        <v>9769.34</v>
+        <v>9521.51</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1493,10 +1501,10 @@
         <v>6</v>
       </c>
       <c r="B4" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="C4" s="3">
-        <v>10291.93</v>
+        <v>10305.93</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1504,10 +1512,10 @@
         <v>7</v>
       </c>
       <c r="B5" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="C5" s="3">
-        <v>1212.72</v>
+        <v>1607.7</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1515,7 +1523,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="C6" s="3">
         <v>89</v>
@@ -1529,7 +1537,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="3">
-        <v>478087912.1</v>
+        <v>475735351.6</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1537,10 +1545,10 @@
         <v>10</v>
       </c>
       <c r="B8" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="C8" s="3">
-        <v>478087912.1</v>
+        <v>475735351.6</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1551,7 +1559,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="3">
-        <v>123591.01</v>
+        <v>117301.06</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1559,7 +1567,7 @@
         <v>12</v>
       </c>
       <c r="B10" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="C10" s="3">
         <v>9529.23</v>
@@ -1570,10 +1578,10 @@
         <v>13</v>
       </c>
       <c r="B11" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="C11" s="3">
-        <v>13643.17</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1581,10 +1589,10 @@
         <v>14</v>
       </c>
       <c r="B12" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="C12" s="4">
-        <v>100418.61</v>
+        <v>100632.3</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1595,7 +1603,7 @@
         <v>4</v>
       </c>
       <c r="C13" s="4">
-        <v>249858380573326</v>
+        <v>248852067055983</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1603,10 +1611,10 @@
         <v>16</v>
       </c>
       <c r="B14" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="C14" s="4">
-        <v>955452490810.13</v>
+        <v>992318745655.99</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1614,10 +1622,10 @@
         <v>17</v>
       </c>
       <c r="B15" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="C15" s="3">
-        <v>248902928082516</v>
+        <v>247859748310328</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1628,7 +1636,7 @@
         <v>4</v>
       </c>
       <c r="C16" s="3">
-        <v>394602.91</v>
+        <v>442667.26</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1636,10 +1644,10 @@
         <v>19</v>
       </c>
       <c r="B17" s="2">
-        <v>403314269</v>
+        <v>410122397</v>
       </c>
       <c r="C17" s="3">
-        <v>394602.91</v>
+        <v>442667.26</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1650,7 +1658,7 @@
         <v>4</v>
       </c>
       <c r="C18" s="3">
-        <v>9956066432.14</v>
+        <v>9956077957.32</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1658,10 +1666,10 @@
         <v>21</v>
       </c>
       <c r="B19" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="C19" s="3">
-        <v>9033592626.19</v>
+        <v>9033604151.38</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1669,7 +1677,7 @@
         <v>22</v>
       </c>
       <c r="B20" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="C20" s="3">
         <v>922473805.94</v>
@@ -1683,7 +1691,7 @@
         <v>4</v>
       </c>
       <c r="C21" s="3">
-        <v>54639062.68</v>
+        <v>237131052.85</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1691,10 +1699,10 @@
         <v>24</v>
       </c>
       <c r="B22" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="C22" s="3">
-        <v>5786173.98</v>
+        <v>8100457.72</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1702,21 +1710,21 @@
         <v>25</v>
       </c>
       <c r="B23" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="C23" s="3">
-        <v>42123888.7</v>
+        <v>229030595.13</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="2">
-        <v>83810027</v>
+      <c r="B24" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="C24" s="3">
-        <v>4895000</v>
+        <v>96023982</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1724,32 +1732,32 @@
         <v>27</v>
       </c>
       <c r="B25" s="2">
-        <v>42686772</v>
+        <v>89830146</v>
       </c>
       <c r="C25" s="3">
-        <v>1834000</v>
+        <v>52334000</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>4</v>
+      <c r="B26" s="2">
+        <v>89830146</v>
       </c>
       <c r="C26" s="3">
-        <v>1208260059.86</v>
+        <v>43689982</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="2">
-        <v>80543001</v>
+      <c r="B27" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="C27" s="3">
-        <v>39211181.7</v>
+        <v>787992072.67</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1757,10 +1765,10 @@
         <v>30</v>
       </c>
       <c r="B28" s="2">
-        <v>79223162</v>
+        <v>81435153</v>
       </c>
       <c r="C28" s="3">
-        <v>190742.36</v>
+        <v>39265232.86</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1768,10 +1776,10 @@
         <v>31</v>
       </c>
       <c r="B29" s="2">
-        <v>24556482</v>
+        <v>81761308</v>
       </c>
       <c r="C29" s="3">
-        <v>100576989.43</v>
+        <v>1254732.6</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1779,10 +1787,10 @@
         <v>32</v>
       </c>
       <c r="B30" s="2">
-        <v>80543001</v>
+        <v>24778642</v>
       </c>
       <c r="C30" s="3">
-        <v>37993772.18</v>
+        <v>32115281.25</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1790,10 +1798,10 @@
         <v>33</v>
       </c>
       <c r="B31" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="C31" s="3">
-        <v>47320569.84</v>
+        <v>87097640.67</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1801,57 +1809,57 @@
         <v>34</v>
       </c>
       <c r="B32" s="2">
-        <v>24355911</v>
+        <v>81435153</v>
       </c>
       <c r="C32" s="3">
-        <v>935450635.64</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
+        <v>17357276.12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B33" s="2">
-        <v>83810027</v>
+        <v>24778642</v>
       </c>
       <c r="C33" s="3">
-        <v>7516168.7</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
+        <v>334402225.53</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B34" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="C34" s="3">
-        <v>40000000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" s="2" t="s">
+        <v>276499683.62</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="5" t="s">
         <v>37</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C35" s="3">
-        <v>33759745.3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
+        <v>32820393.7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B36" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="C36" s="3">
-        <v>33759745.3</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
+        <v>32820393.7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37" s="2" t="s">
         <v>39</v>
       </c>
@@ -1859,78 +1867,60 @@
         <v>4</v>
       </c>
       <c r="C37" s="3">
-        <v>30355740.68</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
+        <v>30851678.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
       <c r="A38" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B38" s="2">
-        <v>102554932</v>
+        <v>103245403</v>
       </c>
       <c r="C38" s="3">
-        <v>30355740.68</v>
+        <v>30851678.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="3">
+        <v>995285</v>
       </c>
     </row>
     <row r="40" spans="1:6">
-      <c r="A40" s="1" t="s">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="2">
+        <v>24778642</v>
+      </c>
+      <c r="C40" s="3">
+        <v>995285</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C40" s="1" t="s">
+      <c r="B42" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B41" s="2" t="s">
+      <c r="E42" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C41" s="2">
-        <v>938735</v>
-      </c>
-      <c r="D41" s="3">
-        <v>7560.7</v>
-      </c>
-      <c r="E41" s="2" t="s">
+      <c r="F42" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C42" s="2">
-        <v>938735</v>
-      </c>
-      <c r="D42" s="3">
-        <v>970.8</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -1938,19 +1928,19 @@
         <v>5</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C43" s="2">
-        <v>938735</v>
+        <v>943083</v>
       </c>
       <c r="D43" s="3">
-        <v>8.38</v>
+        <v>7238.7</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -1958,19 +1948,19 @@
         <v>5</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C44" s="2">
-        <v>938735</v>
+        <v>943083</v>
       </c>
       <c r="D44" s="3">
-        <v>829.68</v>
+        <v>970.79</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -1978,19 +1968,19 @@
         <v>5</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C45" s="2">
-        <v>938735</v>
+        <v>943083</v>
       </c>
       <c r="D45" s="3">
-        <v>80.57</v>
+        <v>8.38</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>4</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -1998,19 +1988,19 @@
         <v>5</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C46" s="2">
+        <v>943083</v>
+      </c>
+      <c r="D46" s="3">
+        <v>829.68</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="C46" s="2">
-        <v>938735</v>
-      </c>
-      <c r="D46" s="3">
-        <v>38.33</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -2018,13 +2008,13 @@
         <v>5</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C47" s="2">
-        <v>938735</v>
+        <v>943083</v>
       </c>
       <c r="D47" s="3">
-        <v>272</v>
+        <v>80.57</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>4</v>
@@ -2038,139 +2028,139 @@
         <v>5</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48" s="2">
+        <v>943083</v>
+      </c>
+      <c r="D48" s="3">
+        <v>38.51</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F48" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="C48" s="2">
-        <v>938735</v>
-      </c>
-      <c r="D48" s="3">
-        <v>8.87</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="C49" s="2">
-        <v>24355911</v>
+        <v>943083</v>
       </c>
       <c r="D49" s="3">
-        <v>1212.72</v>
+        <v>346</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>61</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C50" s="2">
-        <v>80543001</v>
+        <v>943083</v>
       </c>
       <c r="D50" s="3">
-        <v>10208.92</v>
+        <v>8.87</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>63</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="2" t="s">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C51" s="2">
-        <v>80543001</v>
+        <v>24778642</v>
       </c>
       <c r="D51" s="3">
-        <v>83</v>
+        <v>1607.7</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C52" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D52" s="3">
-        <v>89</v>
+        <v>10220.93</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="2" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C53" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D53" s="3">
-        <v>1082075947.73</v>
+        <v>85</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>66</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="2" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C54" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D54" s="3">
-        <v>35318902.35</v>
+        <v>89</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2181,13 +2171,13 @@
         <v>67</v>
       </c>
       <c r="C55" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D55" s="3">
-        <v>1705110564.09</v>
+        <v>1082078671.39</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>68</v>
@@ -2198,19 +2188,19 @@
         <v>21</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C56" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D56" s="3">
-        <v>1434482060.2</v>
+        <v>35318850.32</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -2218,19 +2208,19 @@
         <v>21</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C57" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D57" s="3">
-        <v>1071256469.61</v>
+        <v>1705110564.08</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -2238,19 +2228,19 @@
         <v>21</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C58" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D58" s="3">
-        <v>1070380443.25</v>
+        <v>1434482068.2</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -2258,19 +2248,19 @@
         <v>21</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C59" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D59" s="3">
-        <v>1064078455.88</v>
+        <v>1071260896.39</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -2278,79 +2268,79 @@
         <v>21</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C60" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D60" s="3">
-        <v>1570889775.08</v>
+        <v>1070382146.36</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C61" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D61" s="3">
-        <v>922473805.94</v>
+        <v>1064081179.55</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="C62" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D62" s="2">
-        <v>1060.22</v>
+        <v>81435153</v>
+      </c>
+      <c r="D62" s="3">
+        <v>1570889775.08</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>81</v>
       </c>
       <c r="C63" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D63" s="2">
-        <v>7901.1</v>
+        <v>81435153</v>
+      </c>
+      <c r="D63" s="3">
+        <v>922473805.94</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>4</v>
+        <v>82</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -2358,19 +2348,19 @@
         <v>12</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>4</v>
+        <v>62</v>
+      </c>
+      <c r="C64" s="2">
+        <v>24778642</v>
+      </c>
+      <c r="D64" s="2">
+        <v>160.19</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -2378,19 +2368,19 @@
         <v>12</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>4</v>
+        <v>83</v>
+      </c>
+      <c r="C65" s="2">
+        <v>24778642</v>
+      </c>
+      <c r="D65" s="2">
+        <v>8961.1</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>86</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -2398,7 +2388,7 @@
         <v>12</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>4</v>
@@ -2407,10 +2397,10 @@
         <v>4</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -2418,7 +2408,7 @@
         <v>12</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>4</v>
@@ -2427,10 +2417,10 @@
         <v>4</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -2438,59 +2428,59 @@
         <v>12</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C68" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D68" s="2">
-        <v>567.91</v>
+        <v>89</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="69" spans="1:6">
       <c r="A69" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C69" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D69" s="2">
-        <v>13643.17</v>
+        <v>91</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>61</v>
+        <v>92</v>
       </c>
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>93</v>
       </c>
       <c r="C70" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D70" s="5">
-        <v>28864.52</v>
+        <v>24778642</v>
+      </c>
+      <c r="D70" s="2">
+        <v>547.45</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>4</v>
+        <v>94</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -2498,59 +2488,59 @@
         <v>14</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="C71" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D71" s="5">
-        <v>71554.08</v>
+        <v>24778642</v>
+      </c>
+      <c r="D71" s="2">
+        <v>28925.95</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>61</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:6">
       <c r="A72" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C72" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D72" s="5">
-        <v>343701650000</v>
+        <v>24778642</v>
+      </c>
+      <c r="D72" s="6">
+        <v>71706.36</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="73" spans="1:6">
       <c r="A73" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>91</v>
+        <v>62</v>
       </c>
       <c r="C73" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D73" s="2">
-        <v>11321499172.13</v>
+        <v>24778642</v>
+      </c>
+      <c r="D73" s="6">
+        <v>7000</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>92</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -2558,59 +2548,59 @@
         <v>16</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="C74" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D74" s="2">
-        <v>600429341638</v>
+        <v>24778642</v>
+      </c>
+      <c r="D74" s="6">
+        <v>343701650000</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
     </row>
     <row r="75" spans="1:6">
       <c r="A75" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>4</v>
+        <v>93</v>
+      </c>
+      <c r="C75" s="2">
+        <v>24778642</v>
+      </c>
+      <c r="D75" s="2">
+        <v>11321499172.13</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
     </row>
     <row r="76" spans="1:6">
       <c r="A76" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>4</v>
+        <v>83</v>
+      </c>
+      <c r="C76" s="2">
+        <v>24778642</v>
+      </c>
+      <c r="D76" s="2">
+        <v>600429341638</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>86</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -2618,19 +2608,19 @@
         <v>12</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D77" s="6" t="s">
+      <c r="D77" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -2638,59 +2628,59 @@
         <v>12</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="D78" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="79" spans="1:6">
       <c r="A79" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C79" s="2">
-        <v>80543001</v>
-      </c>
-      <c r="D79" s="5">
-        <v>246698038367579</v>
+        <v>89</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>63</v>
+        <v>90</v>
       </c>
     </row>
     <row r="80" spans="1:6">
       <c r="A80" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C80" s="2">
-        <v>80543001</v>
-      </c>
-      <c r="D80" s="2">
-        <v>2050214000000</v>
+        <v>91</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>4</v>
+        <v>85</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>4</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -2698,33 +2688,33 @@
         <v>17</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>94</v>
+        <v>64</v>
       </c>
       <c r="C81" s="2">
-        <v>80543001</v>
-      </c>
-      <c r="D81" s="2">
-        <v>154675714936.27</v>
+        <v>81435153</v>
+      </c>
+      <c r="D81" s="6">
+        <v>246698038367579</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="C82" s="2">
-        <v>403314269</v>
+        <v>81435153</v>
       </c>
       <c r="D82" s="2">
-        <v>30780.97</v>
+        <v>1000725000000</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>4</v>
@@ -2735,22 +2725,22 @@
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C83" s="2">
+        <v>81435153</v>
+      </c>
+      <c r="D83" s="2">
+        <v>160984942747.81</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F83" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C83" s="2">
-        <v>403314269</v>
-      </c>
-      <c r="D83" s="5">
-        <v>1769.03</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F83" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -2761,10 +2751,10 @@
         <v>98</v>
       </c>
       <c r="C84" s="2">
-        <v>403314269</v>
+        <v>410122397</v>
       </c>
       <c r="D84" s="2">
-        <v>362052.92</v>
+        <v>43480.97</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>4</v>
@@ -2775,36 +2765,36 @@
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C85" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D85" s="2">
-        <v>696173.98</v>
+        <v>410122397</v>
+      </c>
+      <c r="D85" s="6">
+        <v>9480.75</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>92</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="C86" s="2">
-        <v>24556482</v>
+        <v>410122397</v>
       </c>
       <c r="D86" s="2">
-        <v>5090000</v>
+        <v>389705.55</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>4</v>
@@ -2815,96 +2805,96 @@
     </row>
     <row r="87" spans="1:6">
       <c r="A87" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C87" s="2">
-        <v>83810027</v>
+        <v>24778642</v>
       </c>
       <c r="D87" s="2">
-        <v>4895000</v>
+        <v>648457.71</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>4</v>
+        <v>94</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="C88" s="2">
-        <v>24556482</v>
-      </c>
-      <c r="D88" s="5">
-        <v>42123888.7</v>
+        <v>24778642</v>
+      </c>
+      <c r="D88" s="2">
+        <v>7452000</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>61</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="C89" s="2">
-        <v>42686772</v>
+        <v>24778642</v>
       </c>
       <c r="D89" s="2">
-        <v>1834000</v>
+        <v>229030595.13</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C90" s="2">
-        <v>80543001</v>
-      </c>
-      <c r="D90" s="5">
-        <v>39211181.7</v>
+        <v>81435153</v>
+      </c>
+      <c r="D90" s="6">
+        <v>39265232.86</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C91" s="2">
-        <v>79223162</v>
+        <v>81761308</v>
       </c>
       <c r="D91" s="2">
-        <v>190742.36</v>
+        <v>1254732.6</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>4</v>
@@ -2915,22 +2905,22 @@
     </row>
     <row r="92" spans="1:6">
       <c r="A92" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C92" s="2">
-        <v>80543001</v>
-      </c>
-      <c r="D92" s="2">
-        <v>47320569.84</v>
+        <v>81435153</v>
+      </c>
+      <c r="D92" s="6">
+        <v>17357276.12</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -2938,19 +2928,19 @@
         <v>102</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C93" s="2">
         <v>24556482</v>
       </c>
       <c r="D93" s="2">
-        <v>4244576.12</v>
+        <v>3168868.06</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -2967,7 +2957,7 @@
         <v>1045412.19</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>104</v>
@@ -2975,22 +2965,22 @@
     </row>
     <row r="95" spans="1:6">
       <c r="A95" s="2" t="s">
-        <v>102</v>
+        <v>35</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C95" s="2">
         <v>24556482</v>
       </c>
       <c r="D95" s="2">
-        <v>70000000.12</v>
+        <v>334402225.53</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -2998,13 +2988,13 @@
         <v>102</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C96" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="D96" s="2">
-        <v>25287001</v>
+        <v>27901001</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>4</v>
@@ -3018,7 +3008,7 @@
         <v>12</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C97" s="2" t="s">
         <v>4</v>
@@ -3027,10 +3017,10 @@
         <v>4</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -3038,19 +3028,19 @@
         <v>12</v>
       </c>
       <c r="B98" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E98" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C98" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E98" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="F98" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -3058,7 +3048,7 @@
         <v>12</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C99" s="2" t="s">
         <v>4</v>
@@ -3067,10 +3057,10 @@
         <v>4</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -3078,33 +3068,33 @@
         <v>12</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C100" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D100" s="5" t="s">
+      <c r="D100" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="101" spans="1:6">
       <c r="A101" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C101" s="2">
-        <v>80543001</v>
+        <v>81435153</v>
       </c>
       <c r="D101" s="2">
-        <v>32719333.82</v>
+        <v>499640.36</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>4</v>
@@ -3115,7 +3105,7 @@
     </row>
     <row r="102" spans="1:6">
       <c r="A102" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>105</v>
@@ -3123,11 +3113,11 @@
       <c r="C102" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D102" s="2" t="s">
+      <c r="D102" s="6" t="s">
         <v>4</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F102" s="2" t="s">
         <v>106</v>
@@ -3135,7 +3125,7 @@
     </row>
     <row r="103" spans="1:6">
       <c r="A103" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>107</v>
@@ -3147,7 +3137,7 @@
         <v>4</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F103" s="2" t="s">
         <v>108</v>
@@ -3155,7 +3145,7 @@
     </row>
     <row r="104" spans="1:6">
       <c r="A104" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>109</v>
@@ -3163,11 +3153,11 @@
       <c r="C104" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D104" s="3" t="s">
+      <c r="D104" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F104" s="2" t="s">
         <v>110</v>
@@ -3175,102 +3165,102 @@
     </row>
     <row r="105" spans="1:6">
       <c r="A105" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C105" s="2">
         <v>80543001</v>
       </c>
-      <c r="D105" s="3">
+      <c r="D105" s="2">
         <v>3365367.97</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="106" spans="1:6">
       <c r="A106" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C106" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="D106" s="3">
-        <v>935450635.64</v>
+        <v>276499683.62</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>99</v>
+        <v>62</v>
       </c>
       <c r="C107" s="2">
-        <v>83810027</v>
+        <v>89830146</v>
       </c>
       <c r="D107" s="3">
-        <v>7516168.7</v>
+        <v>52334000</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
     </row>
     <row r="108" spans="1:6">
       <c r="A108" s="2" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C108" s="2">
-        <v>24556482</v>
+        <v>89830146</v>
       </c>
       <c r="D108" s="3">
-        <v>40000000</v>
+        <v>43689982</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="109" spans="1:6">
       <c r="A109" s="2" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>111</v>
       </c>
       <c r="C109" s="2">
-        <v>80543001</v>
+        <v>103245403</v>
       </c>
       <c r="D109" s="3">
-        <v>1909070.4</v>
+        <v>28887852.74</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>112</v>
+        <v>4</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -3278,13 +3268,13 @@
         <v>40</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C110" s="2">
-        <v>102554932</v>
+        <v>103245403</v>
       </c>
       <c r="D110" s="3">
-        <v>28087852.73</v>
+        <v>1831000.99</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>4</v>
@@ -3298,13 +3288,13 @@
         <v>40</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C111" s="2">
-        <v>102554932</v>
+        <v>103245403</v>
       </c>
       <c r="D111" s="3">
-        <v>2075001</v>
+        <v>132824.77</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>4</v>
@@ -3315,16 +3305,16 @@
     </row>
     <row r="112" spans="1:6">
       <c r="A112" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>115</v>
+        <v>83</v>
       </c>
       <c r="C112" s="2">
-        <v>102554932</v>
+        <v>24778642</v>
       </c>
       <c r="D112" s="3">
-        <v>192886.95</v>
+        <v>7257000</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>4</v>
@@ -3338,19 +3328,19 @@
         <v>38</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="C113" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="D113" s="3">
-        <v>7257000</v>
+        <v>25156000.02</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -3358,59 +3348,59 @@
         <v>38</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="C114" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="D114" s="3">
-        <v>25156000.02</v>
+        <v>407393.68</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>61</v>
+        <v>94</v>
       </c>
     </row>
     <row r="115" spans="1:6">
       <c r="A115" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C115" s="2">
-        <v>24556482</v>
+        <v>24778642</v>
       </c>
       <c r="D115" s="3">
-        <v>1346745.28</v>
+        <v>686000</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>92</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116" spans="1:6">
       <c r="A116" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="C116" s="2">
-        <v>6104444</v>
+        <v>24778642</v>
       </c>
       <c r="D116" s="3">
-        <v>1209085.000572</v>
+        <v>309285</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>4</v>
+        <v>94</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -3418,13 +3408,13 @@
         <v>10</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C117" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D117" s="3">
-        <v>290913.96752144</v>
+        <v>1039138.48</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>4</v>
@@ -3438,13 +3428,13 @@
         <v>10</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C118" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D118" s="3">
-        <v>364988045.757242</v>
+        <v>319353.64</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>4</v>
@@ -3458,13 +3448,13 @@
         <v>10</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C119" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D119" s="3">
-        <v>17577000.763</v>
+        <v>369891003.49</v>
       </c>
       <c r="E119" s="2" t="s">
         <v>4</v>
@@ -3478,13 +3468,13 @@
         <v>10</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C120" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D120" s="3">
-        <v>66066923.3937279</v>
+        <v>9757000.76</v>
       </c>
       <c r="E120" s="2" t="s">
         <v>4</v>
@@ -3498,13 +3488,13 @@
         <v>10</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C121" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D121" s="3">
-        <v>2866993.9984026</v>
+        <v>66066923.39</v>
       </c>
       <c r="E121" s="2" t="s">
         <v>4</v>
@@ -3518,13 +3508,13 @@
         <v>10</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C122" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D122" s="3">
-        <v>2647816.52635095</v>
+        <v>2866994</v>
       </c>
       <c r="E122" s="2" t="s">
         <v>4</v>
@@ -3538,13 +3528,13 @@
         <v>10</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C123" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D123" s="3">
-        <v>1457329.62563352</v>
+        <v>2647816.53</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>4</v>
@@ -3558,13 +3548,13 @@
         <v>10</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C124" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D124" s="3">
-        <v>1066964.29654224</v>
+        <v>1457329.63</v>
       </c>
       <c r="E124" s="2" t="s">
         <v>4</v>
@@ -3578,13 +3568,13 @@
         <v>10</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C125" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D125" s="3">
-        <v>1063999.813</v>
+        <v>1066964.3</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>4</v>
@@ -3598,13 +3588,13 @@
         <v>10</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C126" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D126" s="3">
-        <v>850746.71291594</v>
+        <v>850746.71</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>4</v>
@@ -3618,13 +3608,13 @@
         <v>10</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C127" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D127" s="3">
-        <v>579364.12614368</v>
+        <v>579364.13</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>4</v>
@@ -3638,13 +3628,13 @@
         <v>10</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C128" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D128" s="3">
-        <v>538350.47626452</v>
+        <v>538350.48</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>4</v>
@@ -3658,13 +3648,13 @@
         <v>10</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C129" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D129" s="3">
-        <v>127419.4406821</v>
+        <v>127419.44</v>
       </c>
       <c r="E129" s="2" t="s">
         <v>4</v>
@@ -3678,13 +3668,13 @@
         <v>10</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C130" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D130" s="3">
-        <v>4212998.542</v>
+        <v>4247999.62</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>4</v>
@@ -3698,13 +3688,13 @@
         <v>10</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C131" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D131" s="3">
-        <v>3388999.664</v>
+        <v>4139999.47</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>4</v>
@@ -3718,13 +3708,13 @@
         <v>10</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C132" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D132" s="3">
-        <v>2871997.347</v>
+        <v>2541998.28</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>4</v>
@@ -3738,13 +3728,13 @@
         <v>10</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C133" s="2">
-        <v>6104444</v>
+        <v>6146643</v>
       </c>
       <c r="D133" s="3">
-        <v>2723999.813</v>
+        <v>1729962.59</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>4</v>
@@ -3758,43 +3748,144 @@
         <v>10</v>
       </c>
       <c r="B134" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C134" s="2">
+        <v>6146643</v>
+      </c>
+      <c r="D134" s="3">
+        <v>1636999.66</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6">
+      <c r="A135" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C135" s="2">
+        <v>6146643</v>
+      </c>
+      <c r="D135" s="3">
+        <v>1150991.11</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6">
+      <c r="A136" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C136" s="2">
+        <v>6146643</v>
+      </c>
+      <c r="D136" s="3">
+        <v>963999.81</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6">
+      <c r="A137" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B137" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C134" s="2">
-        <v>6104444</v>
-      </c>
-      <c r="D134" s="3">
-        <v>1884995.144</v>
-      </c>
-      <c r="E134" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F134" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6">
-      <c r="A135" t="s">
+      <c r="C137" s="2">
+        <v>6146643</v>
+      </c>
+      <c r="D137" s="3">
+        <v>584998.39</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6">
+      <c r="A138" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B138" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C135">
-        <v>6104444</v>
-      </c>
-      <c r="D135">
-        <v>1673967.672</v>
-      </c>
-      <c r="E135" t="s">
-        <v>4</v>
-      </c>
-      <c r="F135" t="s">
+      <c r="C138" s="2">
+        <v>6146643</v>
+      </c>
+      <c r="D138" s="3">
+        <v>553999.81</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6">
+      <c r="A139" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C139" s="2">
+        <v>6146643</v>
+      </c>
+      <c r="D139" s="3">
+        <v>513999.81</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6">
+      <c r="A140" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C140" s="2">
+        <v>6146643</v>
+      </c>
+      <c r="D140" s="3">
+        <v>461998.06</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F140" s="2" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
upgrade: update snapshot 20260601;
</commit_message>
<xml_diff>
--- a/snapshot/huobi_por.xlsx
+++ b/snapshot/huobi_por.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Zhuanz/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A9EEF52-D25F-BC46-BEA3-3231EAE2DBC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83323431-5232-774E-9897-001E66F793B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5520" yWindow="1320" windowWidth="27860" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7800" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="huobi_por" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="145">
   <si>
     <t>coin</t>
   </si>
@@ -56,9 +56,6 @@
     <t>BTC-TRC20</t>
   </si>
   <si>
-    <t>wBTC-ERC20</t>
-  </si>
-  <si>
     <t>jWBTC-TRC20</t>
   </si>
   <si>
@@ -74,9 +71,6 @@
     <t>ETH</t>
   </si>
   <si>
-    <t>Morpho-ETH</t>
-  </si>
-  <si>
     <t>stETH</t>
   </si>
   <si>
@@ -110,9 +104,6 @@
     <t>ERC20-USDC</t>
   </si>
   <si>
-    <t>spUSDC-ERC20</t>
-  </si>
-  <si>
     <t>U(All)</t>
   </si>
   <si>
@@ -137,9 +128,6 @@
     <t>jUSDT-TRC20</t>
   </si>
   <si>
-    <t>spUSDT-ERC20</t>
-  </si>
-  <si>
     <t>USDT-aEthUSDT</t>
   </si>
   <si>
@@ -203,15 +191,9 @@
     <t>H1JDQp1uGjVNXcXdpUUUnbiRS1YyttPeo8btOTuA86tXLEIWrVeoNlZsjufIBkfR/f5wqxklyHg1wnNY3cHqIrw=</t>
   </si>
   <si>
-    <t>3EpyhpDRu2wz5LtS4sPAmXaGozuxYWdRkN</t>
-  </si>
-  <si>
     <t>1JnrLZzvRSc7QngWvQwZjXQ43E1JaYYz2i</t>
   </si>
   <si>
-    <t>WBTC-ERC20</t>
-  </si>
-  <si>
     <t>0x18709e89bd403f470088abdacebe86cc60dda12e</t>
   </si>
   <si>
@@ -371,9 +353,6 @@
     <t>DRRU8L7fF4k9w7SF3Z6ei8onPCsh9hjGX1</t>
   </si>
   <si>
-    <t>9ztZpRN3v9xv5JhAT7MTtmy4DfyMEAG8YU</t>
-  </si>
-  <si>
     <t>DHGb5BKsagXePRWwKqLx2vMH5uUNg8euvN</t>
   </si>
   <si>
@@ -401,27 +380,15 @@
     <t>DB5KWytcxHyphHPn9iC92Y9JqPRL1Fq21p</t>
   </si>
   <si>
-    <t>STEAK-USDC</t>
-  </si>
-  <si>
     <t>BEP20-USDC</t>
   </si>
   <si>
-    <t>USDC-SOL</t>
-  </si>
-  <si>
-    <t>BEP20-ListaU</t>
-  </si>
-  <si>
     <t>TRC20-U</t>
   </si>
   <si>
     <t>USDT-BEP20</t>
   </si>
   <si>
-    <t>USDT-ARC20</t>
-  </si>
-  <si>
     <t>USDS(ALL)</t>
   </si>
   <si>
@@ -452,37 +419,55 @@
     <t>0xafdfd157d9361e621e476036fee62f688450692b</t>
   </si>
   <si>
-    <t>Cw32Ny2xcYdpfJmvFd7h2pRhcbcjoJFq8KrrA8YLwZeh</t>
-  </si>
-  <si>
-    <t>DPqhyyBpjuULZRvdeRwtMMF9JGr1rHjszh</t>
-  </si>
-  <si>
     <t>DL2EGukahtib57Sg7FtHsvf8HgwMJtbBA3</t>
   </si>
   <si>
-    <t>DFfSQtwuHTdHYjtDcxEVj9nkiKRFTDoG6g</t>
-  </si>
-  <si>
-    <t>A2xYv2PujsndgzfUoMexR7hUm3WJRBu11k</t>
-  </si>
-  <si>
-    <t>AAyUiDAt1oPZJMbpg275GnZnqZNyV4Wouj</t>
-  </si>
-  <si>
-    <t>ADjG5rAGmK9wjv8Txfigp5P3N1hHumhLTB</t>
-  </si>
-  <si>
-    <t>9rtihNSbuVykUsXzLtxjuBU6aMW8iHWjwa</t>
-  </si>
-  <si>
-    <t>AADPrD693gq6Mbjy5AgcGAd1otSMiWPte6</t>
-  </si>
-  <si>
-    <t>A5kB2a11h7YcL82GHbxeE2aL62Lk2wHosy</t>
-  </si>
-  <si>
-    <t>9xfk1dj4JXptF15PeQRA46Nz9CdXdKqcPh</t>
+    <t>ThirdParty</t>
+  </si>
+  <si>
+    <t>_</t>
+  </si>
+  <si>
+    <t>TCQQjfccKdMi4CnPAzmZW5TALH4HbwceVb</t>
+  </si>
+  <si>
+    <t>4d3baf9ceb963cb5224005d1f1dc769bbb57c4710ffe5a2432d46c9b8ad22cd90ae94a5f53af14314b68808802aa944a4a99b0c5c181e95b87f32a3f0aeefef700</t>
+  </si>
+  <si>
+    <t>0x3fd039007988ee27acafbf0d3a23734ba7673048</t>
+  </si>
+  <si>
+    <t>0x30741289523c2e4d2a62c7d6722686d14e723851</t>
+  </si>
+  <si>
+    <t>0xd81825f030667d07ed9574e13a93d0dc665c0dd87906e80ed99961569ae064a87268ae621d539f037193bde3ad03a99d6e233e733b59cd79ca7c9d08c12a97a601</t>
+  </si>
+  <si>
+    <t>ERC20-aEthUSDT</t>
+  </si>
+  <si>
+    <t>DJX3kCZfcDuREturnUNKEBQELi1PFaLkJC</t>
+  </si>
+  <si>
+    <t>DLzCvKskasu4Adj3XgbyNitKBukBSa5JPP</t>
+  </si>
+  <si>
+    <t>DRAtyHiqvTrCP4gXKNgrKHKqbRBgdQXQZq</t>
+  </si>
+  <si>
+    <t>9yUrPPjPDo7gjTekQrKERmUgkGUkYTEhyQ</t>
+  </si>
+  <si>
+    <t>A2fSFAHxxd9Je872CHrRHwErXEQXUb8n4Y</t>
+  </si>
+  <si>
+    <t>9veYb4pMuyHL1FfcqGMPzjPZdeF4cTcVp1</t>
+  </si>
+  <si>
+    <t>9u1QQv87QcaJrKxJH1bjnW2hAoXocKGykE</t>
+  </si>
+  <si>
+    <t>9vynXnkugSuN9MtCvgoPbZcysifxwWxVWq</t>
   </si>
 </sst>
 </file>
@@ -490,10 +475,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="180" formatCode="0.00_);[Red]\(0.00\)"/>
-    <numFmt numFmtId="181" formatCode="0.00_ "/>
+    <numFmt numFmtId="176" formatCode="0.00_);[Red]\(0.00\)"/>
+    <numFmt numFmtId="177" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -518,6 +503,14 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="等线"/>
@@ -563,7 +556,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -573,13 +566,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -588,10 +581,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -889,7 +879,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F162"/>
+  <dimension ref="A1:F150"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.1640625" customWidth="1"/>
@@ -919,7 +909,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="3">
-        <v>20837.849999999999</v>
+        <v>20922.77</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -927,10 +917,10 @@
         <v>5</v>
       </c>
       <c r="B3" s="2">
-        <v>947308</v>
+        <v>951871</v>
       </c>
       <c r="C3" s="3">
-        <v>8865.85</v>
+        <v>8691.6</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -938,10 +928,10 @@
         <v>6</v>
       </c>
       <c r="B4" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="C4" s="3">
-        <v>10227.299999999999</v>
+        <v>10422.9</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -949,172 +939,172 @@
         <v>7</v>
       </c>
       <c r="B5" s="2">
-        <v>24993980</v>
+        <v>83191458</v>
       </c>
       <c r="C5" s="3">
-        <v>1655.7</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="2">
-        <v>82298910</v>
+        <v>129</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>130</v>
       </c>
       <c r="C6" s="3">
-        <v>89</v>
+        <v>1719.27</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="3">
-        <v>466458527.35000002</v>
+        <v>454163535.63999999</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" s="2">
-        <v>6187371</v>
+        <v>6229557</v>
       </c>
       <c r="C8" s="3">
-        <v>466458527.35000002</v>
+        <v>454163535.63999999</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="3">
-        <v>118817.9</v>
+        <v>109573.31</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" s="2">
-        <v>24993980</v>
+        <v>25216406</v>
       </c>
       <c r="C10" s="3">
-        <v>10979.49</v>
+        <v>4006.56</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="2">
-        <v>24993980</v>
+        <v>25216406</v>
       </c>
       <c r="C11" s="3">
-        <v>7000</v>
+        <v>29051.02</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="2">
-        <v>24993980</v>
+        <v>129</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>130</v>
       </c>
       <c r="C12" s="4">
-        <v>100838.39999999999</v>
+        <v>76515.73</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C13" s="4">
-        <v>237235983505775</v>
+        <v>235835183039990</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B14" s="2">
-        <v>24993980</v>
+        <v>25216406</v>
       </c>
       <c r="C14" s="4">
-        <v>1017314582572.54</v>
+        <v>1034581507473.59</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B15" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="C15" s="3">
-        <v>236218668923203</v>
+        <v>234800601532516</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="3">
-        <v>448014.89</v>
+        <v>420789.4</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B17" s="2">
-        <v>416689095</v>
+        <v>423406343</v>
       </c>
       <c r="C17" s="3">
-        <v>448014.89</v>
+        <v>420789.4</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C18" s="3">
-        <v>9936133361.3400002</v>
+        <v>9242584856.5300007</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B19" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="C19" s="3">
-        <v>9013659555.3899994</v>
+        <v>8320111050.5900002</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B20" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="C20" s="3">
         <v>922473805.94000006</v>
@@ -1122,357 +1112,399 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C21" s="3">
-        <v>274162978.24000001</v>
+        <v>238931193.18000001</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B22" s="2">
-        <v>24993980</v>
+        <v>25216406</v>
       </c>
       <c r="C22" s="3">
-        <v>30342703.760000002</v>
+        <v>473420.2</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>25</v>
+        <v>115</v>
       </c>
       <c r="B23" s="2">
-        <v>24993980</v>
+        <v>101527929</v>
       </c>
       <c r="C23" s="3">
-        <v>20636493.699999999</v>
+        <v>987263.9</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B24" s="2">
-        <v>24993980</v>
+        <v>129</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>130</v>
       </c>
       <c r="C24" s="3">
-        <v>219380570.44</v>
+        <v>237470509.06999999</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="B25" s="2">
-        <v>95582653</v>
+        <v>23</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="C25" s="3">
-        <v>2142209.4700000002</v>
+        <v>38446011.509999998</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="2" t="s">
-        <v>124</v>
+        <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>416689145</v>
+        <v>101527929</v>
       </c>
       <c r="C26" s="3">
-        <v>1661000.88</v>
+        <v>412000</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>4</v>
+        <v>116</v>
+      </c>
+      <c r="B27" s="2">
+        <v>83191458</v>
       </c>
       <c r="C27" s="3">
-        <v>96348309.109999999</v>
+        <v>20469173.030000001</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="2">
-        <v>95646253</v>
+        <v>129</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>130</v>
       </c>
       <c r="C28" s="3">
-        <v>32334000</v>
+        <v>17564838.48</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="B29" s="2">
-        <v>95646253</v>
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="C29" s="3">
-        <v>43545136.079999998</v>
+        <v>906548772.59000003</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="2" t="s">
-        <v>126</v>
+        <v>26</v>
       </c>
       <c r="B30" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="C30" s="3">
-        <v>20469173.030000001</v>
+        <v>39265232.859999999</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>4</v>
+        <v>27</v>
+      </c>
+      <c r="B31" s="2">
+        <v>86837700</v>
       </c>
       <c r="C31" s="3">
-        <v>1009666376.7</v>
+        <v>613304.94999999995</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B32" s="2">
-        <v>82298910</v>
+        <v>25216406</v>
       </c>
       <c r="C32" s="3">
-        <v>39265232.859999999</v>
+        <v>3609746.46</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B33" s="2">
-        <v>84271850</v>
+        <v>83191458</v>
       </c>
       <c r="C33" s="3">
-        <v>1026269.14</v>
+        <v>2526954</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B34" s="2">
-        <v>24993980</v>
+        <v>83191458</v>
       </c>
       <c r="C34" s="3">
-        <v>111868097.33</v>
+        <v>17357276.120000001</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B35" s="2">
-        <v>82298910</v>
+        <v>25216406</v>
       </c>
       <c r="C35" s="3">
-        <v>28948530.68</v>
+        <v>14303345.08</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="2" t="s">
-        <v>33</v>
+        <v>117</v>
       </c>
       <c r="B36" s="2">
-        <v>82298910</v>
+        <v>101527929</v>
       </c>
       <c r="C36" s="3">
-        <v>17357276.120000001</v>
+        <v>10183407.43</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B37" s="2">
-        <v>24993980</v>
+        <v>129</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>130</v>
       </c>
       <c r="C37" s="3">
-        <v>663186047.85000002</v>
+        <v>818689505.67999995</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B38" s="2">
-        <v>24993980</v>
+        <v>118</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="C38" s="3">
-        <v>20008900.25</v>
+        <v>537679.1</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="2" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B39" s="2">
-        <v>95582653</v>
+        <v>25216406</v>
       </c>
       <c r="C39" s="3">
-        <v>11481500.16</v>
+        <v>537679.1</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B40" s="2">
-        <v>457799023</v>
+        <v>120</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="C40" s="3">
-        <v>3965884.2</v>
+        <v>121569640.87</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>4</v>
+        <v>121</v>
+      </c>
+      <c r="B41" s="2">
+        <v>25216406</v>
       </c>
       <c r="C41" s="3">
-        <v>652679.1</v>
+        <v>44805205.200000003</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="B42" s="2">
-        <v>24993980</v>
+        <v>83191458</v>
       </c>
       <c r="C42" s="3">
-        <v>652679.1</v>
+        <v>297692</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>4</v>
+        <v>123</v>
+      </c>
+      <c r="B43" s="2">
+        <v>83191458</v>
       </c>
       <c r="C43" s="3">
-        <v>129072228.38</v>
+        <v>76466743.670000002</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="B44" s="2">
-        <v>24993980</v>
+        <v>32</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="C44" s="3">
-        <v>40884000</v>
+        <v>25840193.239999998</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="2" t="s">
-        <v>133</v>
+        <v>33</v>
       </c>
       <c r="B45" s="2">
-        <v>82298910</v>
+        <v>25216406</v>
       </c>
       <c r="C45" s="3">
-        <v>11721484.710000001</v>
+        <v>25840193.239999998</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B46" s="2">
-        <v>82298910</v>
+        <v>34</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="C46" s="3">
-        <v>76466743.670000002</v>
+        <v>28857206.899999999</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B47" s="2">
+        <v>104607823</v>
+      </c>
+      <c r="C47" s="3">
+        <v>28857206.899999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C47" s="3">
-        <v>32459666.77</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48" s="2" t="s">
+      <c r="C49" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B48" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="C48" s="3">
-        <v>32459666.77</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6">
-      <c r="A49" s="2" t="s">
+      <c r="F49" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C49" s="3">
-        <v>29372047.739999998</v>
       </c>
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B50" s="2">
-        <v>103915491</v>
-      </c>
-      <c r="C50" s="3">
-        <v>29372047.739999998</v>
+      <c r="C50" s="2">
+        <v>951871</v>
+      </c>
+      <c r="D50" s="3">
+        <v>6752.7</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="51" spans="1:6">
-      <c r="A51" s="8"/>
-      <c r="B51" s="8"/>
-      <c r="C51" s="9"/>
+      <c r="A51" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C51" s="2">
+        <v>951871</v>
+      </c>
+      <c r="D51" s="3">
+        <v>970.8</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C52" s="2">
+        <v>951871</v>
+      </c>
+      <c r="D52" s="3">
+        <v>8.3800000000000008</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="53" spans="1:6">
-      <c r="A53" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B53" s="1" t="s">
+      <c r="A53" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C53" s="2">
+        <v>951871</v>
+      </c>
+      <c r="D53" s="3">
+        <v>829.68</v>
+      </c>
+      <c r="E53" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C53" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>42</v>
+      <c r="F53" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -1480,19 +1512,19 @@
         <v>5</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C54" s="2">
-        <v>947308</v>
+        <v>951871</v>
       </c>
       <c r="D54" s="3">
-        <v>6672.7</v>
+        <v>80.569999999999993</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -1500,19 +1532,19 @@
         <v>5</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C55" s="2">
-        <v>947308</v>
+        <v>951871</v>
       </c>
       <c r="D55" s="3">
-        <v>970.8</v>
+        <v>41.4</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -1520,216 +1552,216 @@
         <v>5</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C56" s="2">
-        <v>947308</v>
+        <v>951871</v>
       </c>
       <c r="D56" s="3">
-        <v>8.3800000000000008</v>
+        <v>8.07</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C57" s="2">
-        <v>947308</v>
+        <v>83191458</v>
       </c>
       <c r="D57" s="3">
-        <v>829.68</v>
+        <v>10313.93</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>53</v>
+        <v>87</v>
       </c>
       <c r="C58" s="2">
-        <v>947308</v>
+        <v>83191458</v>
       </c>
       <c r="D58" s="3">
-        <v>80.569999999999993</v>
+        <v>32.979999999999997</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>4</v>
+        <v>88</v>
       </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C59" s="2">
-        <v>947308</v>
+        <v>83191458</v>
       </c>
       <c r="D59" s="3">
-        <v>19.850000000000001</v>
+        <v>76</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>55</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C60" s="2">
+        <v>83191458</v>
+      </c>
+      <c r="D60" s="3">
+        <v>89</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="C60" s="2">
-        <v>947308</v>
-      </c>
-      <c r="D60" s="3">
-        <v>275</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C61" s="2">
-        <v>947308</v>
+        <v>83191458</v>
       </c>
       <c r="D61" s="3">
-        <v>8.8699999999999992</v>
+        <v>1082083426.3900001</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="2" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>59</v>
+        <v>131</v>
       </c>
       <c r="C62" s="2">
-        <v>24993980</v>
+        <v>83191458</v>
       </c>
       <c r="D62" s="3">
-        <v>1655.7</v>
+        <v>40828.28</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>60</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C63" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="D63" s="3">
-        <v>10223.93</v>
+        <v>478104.22</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>93</v>
+        <v>60</v>
       </c>
       <c r="C64" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="D64" s="3">
-        <v>3.37</v>
+        <v>1705110564.0899999</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>94</v>
+        <v>61</v>
       </c>
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="2" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C65" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="D65" s="3">
-        <v>89</v>
+        <v>755759959.02999997</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="66" spans="1:6">
       <c r="A66" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>64</v>
       </c>
       <c r="C66" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="D66" s="3">
-        <v>1082081079.51</v>
+        <v>1071272981.99</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F66" s="2" t="s">
         <v>65</v>
@@ -1737,262 +1769,262 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C67" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="D67" s="3">
-        <v>15318832.77</v>
+        <v>1070389476.97</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="68" spans="1:6">
       <c r="A68" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C68" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="D68" s="3">
-        <v>1705110564.0799999</v>
+        <v>1064085934.55</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="69" spans="1:6">
       <c r="A69" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C69" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="D69" s="3">
-        <v>1434482068.2</v>
+        <v>1570889775.0799999</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C70" s="2">
-        <v>82298910</v>
+        <v>83191458</v>
       </c>
       <c r="D70" s="3">
-        <v>1071266988.96</v>
+        <v>922473805.94000006</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="71" spans="1:6">
       <c r="A71" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C71" s="2">
-        <v>82298910</v>
-      </c>
-      <c r="D71" s="3">
-        <v>1070385830.83</v>
+        <v>25216406</v>
+      </c>
+      <c r="D71" s="2">
+        <v>3941.1</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>73</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:6">
       <c r="A72" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C72" s="2">
-        <v>82298910</v>
-      </c>
-      <c r="D72" s="3">
-        <v>1064083587.67</v>
+        <v>75</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="73" spans="1:6">
       <c r="A73" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B73" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E73" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C73" s="2">
-        <v>82298910</v>
-      </c>
-      <c r="D73" s="3">
-        <v>1570889775.0799999</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="F73" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="74" spans="1:6">
       <c r="A74" s="2" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C74" s="2">
-        <v>82298910</v>
-      </c>
-      <c r="D74" s="3">
-        <v>922473805.94000006</v>
+        <v>80</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="75" spans="1:6">
       <c r="A75" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C75" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D75" s="2">
-        <v>663.01</v>
+        <v>82</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
     </row>
     <row r="76" spans="1:6">
       <c r="A76" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C76" s="2">
-        <v>24993980</v>
+        <v>25216406</v>
       </c>
       <c r="D76" s="2">
-        <v>9831.1</v>
+        <v>6.6</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>4</v>
+        <v>85</v>
       </c>
     </row>
     <row r="77" spans="1:6">
       <c r="A77" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>4</v>
+        <v>94</v>
+      </c>
+      <c r="C77" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D77" s="2">
+        <v>48.89</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="78" spans="1:6">
       <c r="A78" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>4</v>
+        <v>124</v>
+      </c>
+      <c r="C78" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D78" s="2">
+        <v>5</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>85</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79" spans="1:6">
       <c r="A79" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>4</v>
+        <v>133</v>
+      </c>
+      <c r="C79" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D79" s="5">
+        <v>4.97</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>87</v>
+        <v>4</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -2000,19 +2032,19 @@
         <v>12</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>4</v>
+        <v>86</v>
+      </c>
+      <c r="C80" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D80" s="5">
+        <v>29045.65</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>89</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -2020,59 +2052,59 @@
         <v>12</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>90</v>
+        <v>134</v>
       </c>
       <c r="C81" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D81" s="2">
-        <v>429.64</v>
+        <v>25216406</v>
+      </c>
+      <c r="D81" s="5">
+        <v>5.37</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>91</v>
+        <v>135</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="C82" s="2">
-        <v>24993980</v>
+        <v>25216406</v>
       </c>
       <c r="D82" s="2">
-        <v>48.89</v>
+        <v>386057650000</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>101</v>
+        <v>54</v>
       </c>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>135</v>
+        <v>84</v>
       </c>
       <c r="C83" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D83" s="5">
-        <v>6.85</v>
+        <v>25216406</v>
+      </c>
+      <c r="D83" s="2">
+        <v>15584515835.59</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>4</v>
+        <v>85</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -2080,13 +2112,13 @@
         <v>14</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="C84" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D84" s="5">
-        <v>28985.19</v>
+        <v>25216406</v>
+      </c>
+      <c r="D84" s="2">
+        <v>632939341638</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>4</v>
@@ -2097,182 +2129,182 @@
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C85" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D85" s="5">
-        <v>71853.22</v>
+        <v>75</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C86" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D86" s="2">
-        <v>7000</v>
+        <v>78</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>4</v>
+        <v>79</v>
       </c>
     </row>
     <row r="87" spans="1:6">
       <c r="A87" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C87" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D87" s="2">
-        <v>371580650000</v>
+        <v>80</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D87" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C88" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D88" s="2">
-        <v>12794590934.540001</v>
+        <v>82</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C89" s="2">
-        <v>24993980</v>
+        <v>83191458</v>
       </c>
       <c r="D89" s="2">
-        <v>632939341638</v>
+        <v>234162952118135</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D90" s="6" t="s">
-        <v>4</v>
+        <v>57</v>
+      </c>
+      <c r="C90" s="2">
+        <v>83191458</v>
+      </c>
+      <c r="D90" s="2">
+        <v>271360000000</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>83</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D91" s="5" t="s">
-        <v>4</v>
+        <v>87</v>
+      </c>
+      <c r="C91" s="2">
+        <v>83191458</v>
+      </c>
+      <c r="D91" s="2">
+        <v>366289414380.31</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="92" spans="1:6">
       <c r="A92" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D92" s="5" t="s">
-        <v>4</v>
+        <v>89</v>
+      </c>
+      <c r="C92" s="2">
+        <v>423406343</v>
+      </c>
+      <c r="D92" s="5">
+        <v>5570.97</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>87</v>
+        <v>4</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="A93" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>4</v>
+        <v>90</v>
+      </c>
+      <c r="C93" s="2">
+        <v>423406343</v>
+      </c>
+      <c r="D93" s="2">
+        <v>2421.7600000000002</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>89</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -2280,33 +2312,33 @@
         <v>17</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>61</v>
+        <v>91</v>
       </c>
       <c r="C94" s="2">
-        <v>82298910</v>
+        <v>423406343</v>
       </c>
       <c r="D94" s="2">
-        <v>234672636114058</v>
+        <v>412796.66</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>62</v>
+        <v>4</v>
       </c>
     </row>
     <row r="95" spans="1:6">
       <c r="A95" s="2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="C95" s="2">
-        <v>82298910</v>
+        <v>25216406</v>
       </c>
       <c r="D95" s="2">
-        <v>1391370000000</v>
+        <v>473420.2</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>4</v>
@@ -2317,36 +2349,36 @@
     </row>
     <row r="96" spans="1:6">
       <c r="A96" s="2" t="s">
-        <v>17</v>
+        <v>115</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>93</v>
+        <v>125</v>
       </c>
       <c r="C96" s="2">
-        <v>82298910</v>
-      </c>
-      <c r="D96" s="5">
-        <v>154662809143.89999</v>
+        <v>101527929</v>
+      </c>
+      <c r="D96" s="2">
+        <v>778263.9</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>94</v>
+        <v>126</v>
       </c>
     </row>
     <row r="97" spans="1:6">
       <c r="A97" s="2" t="s">
-        <v>19</v>
+        <v>115</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>95</v>
+        <v>127</v>
       </c>
       <c r="C97" s="2">
-        <v>416689095</v>
-      </c>
-      <c r="D97" s="2">
-        <v>42670.97</v>
+        <v>101527929</v>
+      </c>
+      <c r="D97" s="5">
+        <v>209000</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>4</v>
@@ -2357,36 +2389,36 @@
     </row>
     <row r="98" spans="1:6">
       <c r="A98" s="2" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="C98" s="2">
-        <v>416689095</v>
+        <v>83191458</v>
       </c>
       <c r="D98" s="2">
-        <v>3431.53</v>
+        <v>39265232.859999999</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
     </row>
     <row r="99" spans="1:6">
       <c r="A99" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C99" s="2">
-        <v>416689095</v>
-      </c>
-      <c r="D99" s="2">
-        <v>401912.39</v>
+        <v>86837700</v>
+      </c>
+      <c r="D99" s="5">
+        <v>613304.94999999995</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>4</v>
@@ -2397,76 +2429,76 @@
     </row>
     <row r="100" spans="1:6">
       <c r="A100" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="C100" s="2">
-        <v>24993980</v>
+        <v>83191458</v>
       </c>
       <c r="D100" s="2">
-        <v>2441703.7400000002</v>
+        <v>17357276.120000001</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>91</v>
+        <v>56</v>
       </c>
     </row>
     <row r="101" spans="1:6">
       <c r="A101" s="2" t="s">
-        <v>24</v>
+        <v>93</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C101" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D101" s="5">
-        <v>27901000</v>
+        <v>25216406</v>
+      </c>
+      <c r="D101" s="2">
+        <v>64333.279999999999</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>4</v>
+        <v>85</v>
       </c>
     </row>
     <row r="102" spans="1:6">
       <c r="A102" s="2" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>136</v>
+        <v>94</v>
       </c>
       <c r="C102" s="2">
-        <v>95582653</v>
+        <v>25216406</v>
       </c>
       <c r="D102" s="2">
-        <v>651209.47</v>
+        <v>1045412.19</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
     </row>
     <row r="103" spans="1:6">
       <c r="A103" s="2" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>138</v>
+        <v>74</v>
       </c>
       <c r="C103" s="2">
-        <v>95582653</v>
-      </c>
-      <c r="D103" s="5">
-        <v>1491000</v>
+        <v>25216406</v>
+      </c>
+      <c r="D103" s="2">
+        <v>2500001</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>4</v>
@@ -2477,96 +2509,96 @@
     </row>
     <row r="104" spans="1:6">
       <c r="A104" s="2" t="s">
-        <v>124</v>
+        <v>11</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C104" s="2">
-        <v>416689145</v>
-      </c>
-      <c r="D104" s="2">
-        <v>1661000.88</v>
+        <v>75</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>4</v>
+        <v>77</v>
       </c>
     </row>
     <row r="105" spans="1:6">
       <c r="A105" s="2" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C105" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D105" s="2">
-        <v>20636493.699999999</v>
+        <v>78</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
     </row>
     <row r="106" spans="1:6">
       <c r="A106" s="2" t="s">
-        <v>122</v>
+        <v>11</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C106" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D106" s="2">
-        <v>219380570.44</v>
+        <v>80</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" s="2" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C107" s="2">
-        <v>82298910</v>
-      </c>
-      <c r="D107" s="2">
-        <v>39265232.859999999</v>
+        <v>82</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
     </row>
     <row r="108" spans="1:6">
       <c r="A108" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>98</v>
+        <v>57</v>
       </c>
       <c r="C108" s="2">
-        <v>84271850</v>
+        <v>83191458</v>
       </c>
       <c r="D108" s="2">
-        <v>1026269.14</v>
+        <v>2500000</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>4</v>
@@ -2577,59 +2609,59 @@
     </row>
     <row r="109" spans="1:6">
       <c r="A109" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C109" s="2">
-        <v>82298910</v>
-      </c>
-      <c r="D109" s="2">
-        <v>17357276.120000001</v>
+        <v>96</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>62</v>
+        <v>97</v>
       </c>
     </row>
     <row r="110" spans="1:6">
       <c r="A110" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F110" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="B110" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C110" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D110" s="2">
-        <v>6647684.1500000004</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F110" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="111" spans="1:6">
       <c r="A111" s="2" t="s">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C111" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D111" s="2">
-        <v>1045412.19</v>
+      <c r="C111" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F111" s="2" t="s">
         <v>101</v>
@@ -2637,56 +2669,56 @@
     </row>
     <row r="112" spans="1:6">
       <c r="A112" s="2" t="s">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="C112" s="2">
-        <v>24993980</v>
+        <v>83191458</v>
       </c>
       <c r="D112" s="2">
-        <v>50000000</v>
+        <v>26954</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>60</v>
+        <v>88</v>
       </c>
     </row>
     <row r="113" spans="1:6">
       <c r="A113" s="2" t="s">
-        <v>34</v>
+        <v>136</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="C113" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D113" s="5">
-        <v>663186047.85000002</v>
+        <v>25216406</v>
+      </c>
+      <c r="D113" s="3">
+        <v>14303345.08</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
     </row>
     <row r="114" spans="1:6">
       <c r="A114" s="2" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>80</v>
+        <v>127</v>
       </c>
       <c r="C114" s="2">
-        <v>24993980</v>
-      </c>
-      <c r="D114" s="2">
-        <v>54175001</v>
+        <v>101527929</v>
+      </c>
+      <c r="D114" s="3">
+        <v>4015169.7</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>4</v>
@@ -2697,110 +2729,110 @@
     </row>
     <row r="115" spans="1:6">
       <c r="A115" s="2" t="s">
-        <v>12</v>
+        <v>117</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>4</v>
+        <v>125</v>
+      </c>
+      <c r="C115" s="2">
+        <v>101527929</v>
+      </c>
+      <c r="D115" s="3">
+        <v>6168237.7300000004</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>83</v>
+        <v>126</v>
       </c>
     </row>
     <row r="116" spans="1:6">
       <c r="A116" s="2" t="s">
-        <v>12</v>
+        <v>116</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C116" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D116" s="2" t="s">
-        <v>4</v>
+        <v>57</v>
+      </c>
+      <c r="C116" s="2">
+        <v>83191458</v>
+      </c>
+      <c r="D116" s="3">
+        <v>20469173.030000001</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>85</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117" spans="1:6">
       <c r="A117" s="2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C117" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D117" s="3" t="s">
-        <v>4</v>
+        <v>127</v>
+      </c>
+      <c r="C117" s="2">
+        <v>101527929</v>
+      </c>
+      <c r="D117" s="3">
+        <v>412000</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>87</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118" spans="1:6">
       <c r="A118" s="2" t="s">
-        <v>12</v>
+        <v>119</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C118" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D118" s="3" t="s">
-        <v>4</v>
+        <v>74</v>
+      </c>
+      <c r="C118" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D118" s="3">
+        <v>537679.1</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>89</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119" spans="1:6">
       <c r="A119" s="2" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C119" s="2">
-        <v>82298910</v>
-      </c>
-      <c r="D119" s="3">
-        <v>26881999.309999999</v>
+        <v>75</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>4</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>4</v>
+        <v>77</v>
       </c>
     </row>
     <row r="120" spans="1:6">
       <c r="A120" s="2" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="C120" s="2" t="s">
         <v>4</v>
@@ -2809,18 +2841,18 @@
         <v>4</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
     </row>
     <row r="121" spans="1:6">
       <c r="A121" s="2" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="C121" s="2" t="s">
         <v>4</v>
@@ -2829,18 +2861,18 @@
         <v>4</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>105</v>
+        <v>81</v>
       </c>
     </row>
     <row r="122" spans="1:6">
       <c r="A122" s="2" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="C122" s="2" t="s">
         <v>4</v>
@@ -2849,104 +2881,104 @@
         <v>4</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
     </row>
     <row r="123" spans="1:6">
       <c r="A123" s="2" t="s">
-        <v>32</v>
+        <v>121</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="C123" s="2">
-        <v>82298910</v>
+        <v>25216406</v>
       </c>
       <c r="D123" s="3">
-        <v>2066531.37</v>
+        <v>44805205.200000003</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>94</v>
+        <v>54</v>
       </c>
     </row>
     <row r="124" spans="1:6">
       <c r="A124" s="2" t="s">
-        <v>35</v>
+        <v>122</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C124" s="2">
-        <v>24993980</v>
+        <v>83191458</v>
       </c>
       <c r="D124" s="3">
-        <v>20008900.25</v>
+        <v>297692</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="125" spans="1:6">
       <c r="A125" s="2" t="s">
-        <v>27</v>
+        <v>123</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C125" s="2">
-        <v>95646253</v>
+        <v>83191458</v>
       </c>
       <c r="D125" s="3">
-        <v>32334000</v>
+        <v>76466743.670000002</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="126" spans="1:6">
       <c r="A126" s="2" t="s">
-        <v>125</v>
+        <v>35</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>59</v>
+        <v>102</v>
       </c>
       <c r="C126" s="2">
-        <v>95646253</v>
+        <v>104607823</v>
       </c>
       <c r="D126" s="3">
-        <v>43545136.079999998</v>
+        <v>27987852.739999998</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127" spans="1:6">
       <c r="A127" s="2" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>63</v>
+        <v>103</v>
       </c>
       <c r="C127" s="2">
-        <v>82298910</v>
+        <v>104607823</v>
       </c>
       <c r="D127" s="3">
-        <v>20469173.030000001</v>
+        <v>766000.99</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>4</v>
@@ -2957,16 +2989,16 @@
     </row>
     <row r="128" spans="1:6">
       <c r="A128" s="2" t="s">
-        <v>130</v>
+        <v>35</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="C128" s="2">
-        <v>24993980</v>
+        <v>104607823</v>
       </c>
       <c r="D128" s="3">
-        <v>652679.1</v>
+        <v>103353.17</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>4</v>
@@ -2977,156 +3009,156 @@
     </row>
     <row r="129" spans="1:6">
       <c r="A129" s="2" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C129" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D129" s="3" t="s">
-        <v>4</v>
+        <v>74</v>
+      </c>
+      <c r="C129" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D129" s="3">
+        <v>10000000</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>83</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130" spans="1:6">
       <c r="A130" s="2" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C130" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D130" s="3" t="s">
-        <v>4</v>
+        <v>53</v>
+      </c>
+      <c r="C130" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D130" s="3">
+        <v>15156000.02</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>85</v>
+        <v>54</v>
       </c>
     </row>
     <row r="131" spans="1:6">
       <c r="A131" s="2" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C131" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D131" s="3" t="s">
-        <v>4</v>
+        <v>84</v>
+      </c>
+      <c r="C131" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D131" s="3">
+        <v>684193.22</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="132" spans="1:6">
       <c r="A132" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C132" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D132" s="3" t="s">
-        <v>4</v>
+        <v>137</v>
+      </c>
+      <c r="C132" s="2">
+        <v>6229557</v>
+      </c>
+      <c r="D132" s="3">
+        <v>268855.80028187</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>89</v>
+        <v>4</v>
       </c>
     </row>
     <row r="133" spans="1:6">
       <c r="A133" s="2" t="s">
-        <v>132</v>
+        <v>9</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>59</v>
+        <v>128</v>
       </c>
       <c r="C133" s="2">
-        <v>24993980</v>
+        <v>6229557</v>
       </c>
       <c r="D133" s="3">
-        <v>40884000</v>
+        <v>187180.2115</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F133" s="2" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
     </row>
     <row r="134" spans="1:6">
       <c r="A134" s="2" t="s">
-        <v>133</v>
+        <v>9</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>61</v>
+        <v>138</v>
       </c>
       <c r="C134" s="2">
-        <v>82298910</v>
+        <v>6229557</v>
       </c>
       <c r="D134" s="3">
-        <v>11721484.710000001</v>
+        <v>156897.95726011001</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F134" s="2" t="s">
-        <v>62</v>
+        <v>4</v>
       </c>
     </row>
     <row r="135" spans="1:6">
       <c r="A135" s="2" t="s">
-        <v>134</v>
+        <v>9</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>61</v>
+        <v>105</v>
       </c>
       <c r="C135" s="2">
-        <v>82298910</v>
+        <v>6229557</v>
       </c>
       <c r="D135" s="3">
-        <v>76466743.670000002</v>
+        <v>369891003.48900002</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>62</v>
+        <v>4</v>
       </c>
     </row>
     <row r="136" spans="1:6">
-      <c r="A136" s="2" t="s">
-        <v>39</v>
+      <c r="A136" s="8" t="s">
+        <v>9</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C136" s="2">
-        <v>103915491</v>
+        <v>6229557</v>
       </c>
       <c r="D136" s="3">
-        <v>27387852.739999998</v>
+        <v>66066923.393727899</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>4</v>
@@ -3137,16 +3169,16 @@
     </row>
     <row r="137" spans="1:6">
       <c r="A137" s="2" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C137" s="2">
-        <v>103915491</v>
+        <v>6229557</v>
       </c>
       <c r="D137" s="3">
-        <v>1893000.99</v>
+        <v>2866993.9984026002</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>4</v>
@@ -3157,16 +3189,16 @@
     </row>
     <row r="138" spans="1:6">
       <c r="A138" s="2" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C138" s="2">
-        <v>103915491</v>
+        <v>6229557</v>
       </c>
       <c r="D138" s="3">
-        <v>91194</v>
+        <v>2647816.5263509499</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>4</v>
@@ -3177,16 +3209,16 @@
     </row>
     <row r="139" spans="1:6">
       <c r="A139" s="2" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="C139" s="2">
-        <v>24993980</v>
+        <v>6229557</v>
       </c>
       <c r="D139" s="3">
-        <v>6957000</v>
+        <v>1457329.6256335201</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>4</v>
@@ -3197,56 +3229,56 @@
     </row>
     <row r="140" spans="1:6">
       <c r="A140" s="2" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>59</v>
+        <v>110</v>
       </c>
       <c r="C140" s="2">
-        <v>24993980</v>
+        <v>6229557</v>
       </c>
       <c r="D140" s="3">
-        <v>25156000.02</v>
+        <v>1066964.2965422401</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
     </row>
     <row r="141" spans="1:6">
       <c r="A141" s="2" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="C141" s="2">
-        <v>24993980</v>
+        <v>6229557</v>
       </c>
       <c r="D141" s="3">
-        <v>346666.75</v>
+        <v>850746.71291593998</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>91</v>
+        <v>4</v>
       </c>
     </row>
     <row r="142" spans="1:6">
       <c r="A142" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="C142" s="2">
-        <v>6187371</v>
+        <v>6229557</v>
       </c>
       <c r="D142" s="3">
-        <v>175145.03273599001</v>
+        <v>579364.12614367995</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>4</v>
@@ -3257,16 +3289,16 @@
     </row>
     <row r="143" spans="1:6">
       <c r="A143" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>141</v>
+        <v>113</v>
       </c>
       <c r="C143" s="2">
-        <v>6187371</v>
+        <v>6229557</v>
       </c>
       <c r="D143" s="3">
-        <v>237999.03748734001</v>
+        <v>538350.47626451997</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>4</v>
@@ -3277,16 +3309,16 @@
     </row>
     <row r="144" spans="1:6">
       <c r="A144" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>142</v>
+        <v>114</v>
       </c>
       <c r="C144" s="2">
-        <v>6187371</v>
+        <v>6229557</v>
       </c>
       <c r="D144" s="3">
-        <v>267511.09999999998</v>
+        <v>127419.4406821</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>4</v>
@@ -3297,16 +3329,16 @@
     </row>
     <row r="145" spans="1:6">
       <c r="A145" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>111</v>
+        <v>139</v>
       </c>
       <c r="C145" s="2">
-        <v>6187371</v>
+        <v>6229557</v>
       </c>
       <c r="D145" s="3">
-        <v>369891003.48900002</v>
+        <v>104766.0303</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>4</v>
@@ -3317,16 +3349,16 @@
     </row>
     <row r="146" spans="1:6">
       <c r="A146" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>112</v>
+        <v>140</v>
       </c>
       <c r="C146" s="2">
-        <v>6187371</v>
+        <v>6229557</v>
       </c>
       <c r="D146" s="3">
-        <v>8527000.7640000004</v>
+        <v>4535998.9539999999</v>
       </c>
       <c r="E146" s="2" t="s">
         <v>4</v>
@@ -3337,16 +3369,16 @@
     </row>
     <row r="147" spans="1:6">
       <c r="A147" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>113</v>
+        <v>141</v>
       </c>
       <c r="C147" s="2">
-        <v>6187371</v>
+        <v>6229557</v>
       </c>
       <c r="D147" s="3">
-        <v>66686944.863125503</v>
+        <v>1054996.6370000001</v>
       </c>
       <c r="E147" s="2" t="s">
         <v>4</v>
@@ -3357,16 +3389,16 @@
     </row>
     <row r="148" spans="1:6">
       <c r="A148" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>114</v>
+        <v>142</v>
       </c>
       <c r="C148" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D148" s="3">
-        <v>2866993.9984026002</v>
+        <v>6229557</v>
+      </c>
+      <c r="D148" s="2">
+        <v>1018930.2</v>
       </c>
       <c r="E148" s="2" t="s">
         <v>4</v>
@@ -3377,16 +3409,16 @@
     </row>
     <row r="149" spans="1:6">
       <c r="A149" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="C149" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D149" s="3">
-        <v>2647816.5263509499</v>
+        <v>6229557</v>
+      </c>
+      <c r="D149" s="2">
+        <v>497999.43900000001</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>4</v>
@@ -3397,261 +3429,21 @@
     </row>
     <row r="150" spans="1:6">
       <c r="A150" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>116</v>
+        <v>144</v>
       </c>
       <c r="C150" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D150" s="3">
-        <v>1457329.6256335201</v>
+        <v>6229557</v>
+      </c>
+      <c r="D150" s="2">
+        <v>244998.32</v>
       </c>
       <c r="E150" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F150" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6">
-      <c r="A151" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B151" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C151" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D151" s="3">
-        <v>1066964.2965422401</v>
-      </c>
-      <c r="E151" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F151" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6">
-      <c r="A152" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B152" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C152" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D152" s="2">
-        <v>850746.71291593998</v>
-      </c>
-      <c r="E152" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F152" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="153" spans="1:6">
-      <c r="A153" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B153" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C153" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D153" s="2">
-        <v>579364.12614367995</v>
-      </c>
-      <c r="E153" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F153" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6">
-      <c r="A154" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B154" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C154" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D154" s="2">
-        <v>538350.47626451997</v>
-      </c>
-      <c r="E154" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F154" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="155" spans="1:6">
-      <c r="A155" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B155" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C155" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D155" s="2">
-        <v>127419.4406821</v>
-      </c>
-      <c r="E155" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F155" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="156" spans="1:6">
-      <c r="A156" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B156" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C156" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D156" s="2">
-        <v>5661981.1720000003</v>
-      </c>
-      <c r="E156" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F156" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="157" spans="1:6">
-      <c r="A157" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B157" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="C157" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D157" s="2">
-        <v>1834957.621</v>
-      </c>
-      <c r="E157" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F157" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="158" spans="1:6">
-      <c r="A158" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B158" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C158" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D158" s="2">
-        <v>1072999.8130000001</v>
-      </c>
-      <c r="E158" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F158" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="159" spans="1:6">
-      <c r="A159" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B159" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C159" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D159" s="2">
-        <v>787999.81299999997</v>
-      </c>
-      <c r="E159" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F159" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="160" spans="1:6">
-      <c r="A160" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B160" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C160" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D160" s="2">
-        <v>437999.81300000002</v>
-      </c>
-      <c r="E160" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F160" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="161" spans="1:6">
-      <c r="A161" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B161" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="C161" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D161" s="2">
-        <v>372999.81300000002</v>
-      </c>
-      <c r="E161" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F161" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="162" spans="1:6">
-      <c r="A162" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B162" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="C162" s="2">
-        <v>6187371</v>
-      </c>
-      <c r="D162" s="2">
-        <v>368999.81300000002</v>
-      </c>
-      <c r="E162" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F162" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
upgrade: upgrade to version 1.7.1
</commit_message>
<xml_diff>
--- a/snapshot/huobi_por.xlsx
+++ b/snapshot/huobi_por.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Zhuanz/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Zhuanz/Desktop/merkle07/Tool-Node.js-VerifyAddress/snapshot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83323431-5232-774E-9897-001E66F793B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95D8BD2D-CF54-354D-B70D-E7289886CAF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7800" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7180" yWindow="1580" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="huobi_por" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="144">
   <si>
     <t>coin</t>
   </si>
@@ -345,9 +345,6 @@
   </si>
   <si>
     <t>rPzT7GA6vWU3PvYSXBpdP5fQPnzwVLwL24</t>
-  </si>
-  <si>
-    <t>rneMKXXdKMD1R9WZ4Yqv1bfst6bjpaD5tP</t>
   </si>
   <si>
     <t>DRRU8L7fF4k9w7SF3Z6ei8onPCsh9hjGX1</t>
@@ -879,7 +876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F150"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.1640625" customWidth="1"/>
@@ -947,10 +944,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="C6" s="3">
         <v>1719.27</v>
@@ -1013,10 +1010,10 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="C12" s="4">
         <v>76515.73</v>
@@ -1134,7 +1131,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B23" s="2">
         <v>101527929</v>
@@ -1145,10 +1142,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="C24" s="3">
         <v>237470509.06999999</v>
@@ -1178,7 +1175,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B27" s="2">
         <v>83191458</v>
@@ -1189,10 +1186,10 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="C28" s="3">
         <v>17564838.48</v>
@@ -1277,7 +1274,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B36" s="2">
         <v>101527929</v>
@@ -1288,10 +1285,10 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="C37" s="3">
         <v>818689505.67999995</v>
@@ -1299,7 +1296,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>4</v>
@@ -1310,7 +1307,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B39" s="2">
         <v>25216406</v>
@@ -1321,7 +1318,7 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>4</v>
@@ -1332,7 +1329,7 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B41" s="2">
         <v>25216406</v>
@@ -1343,7 +1340,7 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B42" s="2">
         <v>83191458</v>
@@ -1354,7 +1351,7 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B43" s="2">
         <v>83191458</v>
@@ -1393,7 +1390,7 @@
         <v>4</v>
       </c>
       <c r="C46" s="3">
-        <v>28857206.899999999</v>
+        <v>28753853.73</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1404,7 +1401,7 @@
         <v>104607823</v>
       </c>
       <c r="C47" s="3">
-        <v>28857206.899999999</v>
+        <v>28753853.73</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -1672,7 +1669,7 @@
         <v>19</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C62" s="2">
         <v>83191458</v>
@@ -1684,7 +1681,7 @@
         <v>40</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -1992,7 +1989,7 @@
         <v>11</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C78" s="2">
         <v>25216406</v>
@@ -2012,7 +2009,7 @@
         <v>11</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C79" s="2">
         <v>25216406</v>
@@ -2052,7 +2049,7 @@
         <v>12</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C81" s="2">
         <v>25216406</v>
@@ -2064,7 +2061,7 @@
         <v>45</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -2349,10 +2346,10 @@
     </row>
     <row r="96" spans="1:6">
       <c r="A96" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C96" s="2">
         <v>101527929</v>
@@ -2364,15 +2361,15 @@
         <v>45</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="97" spans="1:6">
       <c r="A97" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C97" s="2">
         <v>101527929</v>
@@ -2689,7 +2686,7 @@
     </row>
     <row r="113" spans="1:6">
       <c r="A113" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>74</v>
@@ -2709,10 +2706,10 @@
     </row>
     <row r="114" spans="1:6">
       <c r="A114" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C114" s="2">
         <v>101527929</v>
@@ -2729,10 +2726,10 @@
     </row>
     <row r="115" spans="1:6">
       <c r="A115" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C115" s="2">
         <v>101527929</v>
@@ -2744,12 +2741,12 @@
         <v>45</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="116" spans="1:6">
       <c r="A116" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>57</v>
@@ -2772,7 +2769,7 @@
         <v>24</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C117" s="2">
         <v>101527929</v>
@@ -2789,7 +2786,7 @@
     </row>
     <row r="118" spans="1:6">
       <c r="A118" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>74</v>
@@ -2889,7 +2886,7 @@
     </row>
     <row r="123" spans="1:6">
       <c r="A123" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>53</v>
@@ -2909,7 +2906,7 @@
     </row>
     <row r="124" spans="1:6">
       <c r="A124" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>55</v>
@@ -2929,7 +2926,7 @@
     </row>
     <row r="125" spans="1:6">
       <c r="A125" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>55</v>
@@ -2989,16 +2986,16 @@
     </row>
     <row r="128" spans="1:6">
       <c r="A128" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="C128" s="2">
-        <v>104607823</v>
+        <v>25216406</v>
       </c>
       <c r="D128" s="3">
-        <v>103353.17</v>
+        <v>10000000</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>4</v>
@@ -3012,19 +3009,19 @@
         <v>33</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="C129" s="2">
         <v>25216406</v>
       </c>
       <c r="D129" s="3">
-        <v>10000000</v>
+        <v>15156000.02</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>4</v>
+        <v>54</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -3032,39 +3029,39 @@
         <v>33</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="C130" s="2">
         <v>25216406</v>
       </c>
       <c r="D130" s="3">
-        <v>15156000.02</v>
+        <v>684193.22</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
     </row>
     <row r="131" spans="1:6">
       <c r="A131" s="2" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>84</v>
+        <v>136</v>
       </c>
       <c r="C131" s="2">
-        <v>25216406</v>
+        <v>6229557</v>
       </c>
       <c r="D131" s="3">
-        <v>684193.22</v>
+        <v>268855.80028187</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>85</v>
+        <v>4</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -3072,13 +3069,13 @@
         <v>9</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C132" s="2">
         <v>6229557</v>
       </c>
       <c r="D132" s="3">
-        <v>268855.80028187</v>
+        <v>187180.2115</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>4</v>
@@ -3092,13 +3089,13 @@
         <v>9</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="C133" s="2">
         <v>6229557</v>
       </c>
       <c r="D133" s="3">
-        <v>187180.2115</v>
+        <v>156897.95726011001</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>4</v>
@@ -3112,13 +3109,13 @@
         <v>9</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>138</v>
+        <v>104</v>
       </c>
       <c r="C134" s="2">
         <v>6229557</v>
       </c>
       <c r="D134" s="3">
-        <v>156897.95726011001</v>
+        <v>369891003.48900002</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>4</v>
@@ -3128,7 +3125,7 @@
       </c>
     </row>
     <row r="135" spans="1:6">
-      <c r="A135" s="2" t="s">
+      <c r="A135" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B135" s="2" t="s">
@@ -3138,7 +3135,7 @@
         <v>6229557</v>
       </c>
       <c r="D135" s="3">
-        <v>369891003.48900002</v>
+        <v>66066923.393727899</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>4</v>
@@ -3148,7 +3145,7 @@
       </c>
     </row>
     <row r="136" spans="1:6">
-      <c r="A136" s="8" t="s">
+      <c r="A136" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B136" s="2" t="s">
@@ -3158,7 +3155,7 @@
         <v>6229557</v>
       </c>
       <c r="D136" s="3">
-        <v>66066923.393727899</v>
+        <v>2866993.9984026002</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>4</v>
@@ -3178,7 +3175,7 @@
         <v>6229557</v>
       </c>
       <c r="D137" s="3">
-        <v>2866993.9984026002</v>
+        <v>2647816.5263509499</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>4</v>
@@ -3198,7 +3195,7 @@
         <v>6229557</v>
       </c>
       <c r="D138" s="3">
-        <v>2647816.5263509499</v>
+        <v>1457329.6256335201</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>4</v>
@@ -3218,7 +3215,7 @@
         <v>6229557</v>
       </c>
       <c r="D139" s="3">
-        <v>1457329.6256335201</v>
+        <v>1066964.2965422401</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>4</v>
@@ -3238,7 +3235,7 @@
         <v>6229557</v>
       </c>
       <c r="D140" s="3">
-        <v>1066964.2965422401</v>
+        <v>850746.71291593998</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>4</v>
@@ -3258,7 +3255,7 @@
         <v>6229557</v>
       </c>
       <c r="D141" s="3">
-        <v>850746.71291593998</v>
+        <v>579364.12614367995</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>4</v>
@@ -3278,7 +3275,7 @@
         <v>6229557</v>
       </c>
       <c r="D142" s="3">
-        <v>579364.12614367995</v>
+        <v>538350.47626451997</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>4</v>
@@ -3298,7 +3295,7 @@
         <v>6229557</v>
       </c>
       <c r="D143" s="3">
-        <v>538350.47626451997</v>
+        <v>127419.4406821</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>4</v>
@@ -3312,13 +3309,13 @@
         <v>9</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="C144" s="2">
         <v>6229557</v>
       </c>
       <c r="D144" s="3">
-        <v>127419.4406821</v>
+        <v>104766.0303</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>4</v>
@@ -3338,7 +3335,7 @@
         <v>6229557</v>
       </c>
       <c r="D145" s="3">
-        <v>104766.0303</v>
+        <v>4535998.9539999999</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>4</v>
@@ -3358,7 +3355,7 @@
         <v>6229557</v>
       </c>
       <c r="D146" s="3">
-        <v>4535998.9539999999</v>
+        <v>1054996.6370000001</v>
       </c>
       <c r="E146" s="2" t="s">
         <v>4</v>
@@ -3377,8 +3374,8 @@
       <c r="C147" s="2">
         <v>6229557</v>
       </c>
-      <c r="D147" s="3">
-        <v>1054996.6370000001</v>
+      <c r="D147" s="2">
+        <v>1018930.2</v>
       </c>
       <c r="E147" s="2" t="s">
         <v>4</v>
@@ -3398,7 +3395,7 @@
         <v>6229557</v>
       </c>
       <c r="D148" s="2">
-        <v>1018930.2</v>
+        <v>497999.43900000001</v>
       </c>
       <c r="E148" s="2" t="s">
         <v>4</v>
@@ -3418,32 +3415,12 @@
         <v>6229557</v>
       </c>
       <c r="D149" s="2">
-        <v>497999.43900000001</v>
+        <v>244998.32</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F149" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6">
-      <c r="A150" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B150" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="C150" s="2">
-        <v>6229557</v>
-      </c>
-      <c r="D150" s="2">
-        <v>244998.32</v>
-      </c>
-      <c r="E150" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F150" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
upgrade: upgrade to version 1.7.2
</commit_message>
<xml_diff>
--- a/snapshot/huobi_por.xlsx
+++ b/snapshot/huobi_por.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Zhuanz/Desktop/merkle07/Tool-Node.js-VerifyAddress/snapshot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95D8BD2D-CF54-354D-B70D-E7289886CAF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C08A825-B9AD-1B43-8D53-A61E0D09A014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7180" yWindow="1580" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12700" yWindow="2160" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="huobi_por" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="143">
   <si>
     <t>coin</t>
   </si>
@@ -189,9 +189,6 @@
   </si>
   <si>
     <t>H1JDQp1uGjVNXcXdpUUUnbiRS1YyttPeo8btOTuA86tXLEIWrVeoNlZsjufIBkfR/f5wqxklyHg1wnNY3cHqIrw=</t>
-  </si>
-  <si>
-    <t>1JnrLZzvRSc7QngWvQwZjXQ43E1JaYYz2i</t>
   </si>
   <si>
     <t>0x18709e89bd403f470088abdacebe86cc60dda12e</t>
@@ -876,7 +873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F149"/>
+  <dimension ref="A1:F148"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.1640625" customWidth="1"/>
@@ -906,7 +903,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="3">
-        <v>20922.77</v>
+        <v>20914.7</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -917,7 +914,7 @@
         <v>951871</v>
       </c>
       <c r="C3" s="3">
-        <v>8691.6</v>
+        <v>8683.5300000000007</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -944,10 +941,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="C6" s="3">
         <v>1719.27</v>
@@ -1010,10 +1007,10 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="C12" s="4">
         <v>76515.73</v>
@@ -1131,7 +1128,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B23" s="2">
         <v>101527929</v>
@@ -1142,10 +1139,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="C24" s="3">
         <v>237470509.06999999</v>
@@ -1175,7 +1172,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B27" s="2">
         <v>83191458</v>
@@ -1186,10 +1183,10 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="C28" s="3">
         <v>17564838.48</v>
@@ -1274,7 +1271,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B36" s="2">
         <v>101527929</v>
@@ -1285,10 +1282,10 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="C37" s="3">
         <v>818689505.67999995</v>
@@ -1296,7 +1293,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>4</v>
@@ -1307,7 +1304,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B39" s="2">
         <v>25216406</v>
@@ -1318,7 +1315,7 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>4</v>
@@ -1329,7 +1326,7 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B41" s="2">
         <v>25216406</v>
@@ -1340,7 +1337,7 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B42" s="2">
         <v>83191458</v>
@@ -1351,7 +1348,7 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B43" s="2">
         <v>83191458</v>
@@ -1546,22 +1543,22 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C56" s="2">
-        <v>951871</v>
+        <v>83191458</v>
       </c>
       <c r="D56" s="3">
-        <v>8.07</v>
+        <v>10313.93</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -1569,19 +1566,19 @@
         <v>6</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="C57" s="2">
         <v>83191458</v>
       </c>
       <c r="D57" s="3">
-        <v>10313.93</v>
+        <v>32.979999999999997</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -1589,59 +1586,59 @@
         <v>6</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="C58" s="2">
         <v>83191458</v>
       </c>
       <c r="D58" s="3">
-        <v>32.979999999999997</v>
+        <v>76</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>88</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C59" s="2">
         <v>83191458</v>
       </c>
       <c r="D59" s="3">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C60" s="2">
         <v>83191458</v>
       </c>
       <c r="D60" s="3">
-        <v>89</v>
+        <v>1082083426.3900001</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -1649,19 +1646,19 @@
         <v>19</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>58</v>
+        <v>129</v>
       </c>
       <c r="C61" s="2">
         <v>83191458</v>
       </c>
       <c r="D61" s="3">
-        <v>1082083426.3900001</v>
+        <v>40828.28</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>59</v>
+        <v>130</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -1669,19 +1666,19 @@
         <v>19</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>130</v>
+        <v>54</v>
       </c>
       <c r="C62" s="2">
         <v>83191458</v>
       </c>
       <c r="D62" s="3">
-        <v>40828.28</v>
+        <v>478104.22</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -1689,19 +1686,19 @@
         <v>19</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C63" s="2">
         <v>83191458</v>
       </c>
       <c r="D63" s="3">
-        <v>478104.22</v>
+        <v>1705110564.0899999</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -1709,19 +1706,19 @@
         <v>19</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C64" s="2">
         <v>83191458</v>
       </c>
       <c r="D64" s="3">
-        <v>1705110564.0899999</v>
+        <v>755759959.02999997</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -1729,19 +1726,19 @@
         <v>19</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C65" s="2">
         <v>83191458</v>
       </c>
       <c r="D65" s="3">
-        <v>755759959.02999997</v>
+        <v>1071272981.99</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -1749,19 +1746,19 @@
         <v>19</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C66" s="2">
         <v>83191458</v>
       </c>
       <c r="D66" s="3">
-        <v>1071272981.99</v>
+        <v>1070389476.97</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -1769,19 +1766,19 @@
         <v>19</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C67" s="2">
         <v>83191458</v>
       </c>
       <c r="D67" s="3">
-        <v>1070389476.97</v>
+        <v>1064085934.55</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -1789,59 +1786,59 @@
         <v>19</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C68" s="2">
         <v>83191458</v>
       </c>
       <c r="D68" s="3">
-        <v>1064085934.55</v>
+        <v>1570889775.0799999</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="69" spans="1:6">
       <c r="A69" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C69" s="2">
         <v>83191458</v>
       </c>
       <c r="D69" s="3">
-        <v>1570889775.0799999</v>
+        <v>922473805.94000006</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="2" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C70" s="2">
-        <v>83191458</v>
-      </c>
-      <c r="D70" s="3">
-        <v>922473805.94000006</v>
+        <v>25216406</v>
+      </c>
+      <c r="D70" s="2">
+        <v>3941.1</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>73</v>
+        <v>4</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -1851,17 +1848,17 @@
       <c r="B71" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C71" s="2">
-        <v>25216406</v>
-      </c>
-      <c r="D71" s="2">
-        <v>3941.1</v>
+      <c r="C71" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -1869,19 +1866,19 @@
         <v>11</v>
       </c>
       <c r="B72" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E72" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C72" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="F72" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -1889,7 +1886,7 @@
         <v>11</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>4</v>
@@ -1898,10 +1895,10 @@
         <v>4</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -1909,7 +1906,7 @@
         <v>11</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C74" s="2" t="s">
         <v>4</v>
@@ -1918,10 +1915,10 @@
         <v>4</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -1929,19 +1926,19 @@
         <v>11</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>4</v>
+        <v>83</v>
+      </c>
+      <c r="C75" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D75" s="2">
+        <v>6.6</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -1949,19 +1946,19 @@
         <v>11</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="C76" s="2">
         <v>25216406</v>
       </c>
       <c r="D76" s="2">
-        <v>6.6</v>
+        <v>48.89</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -1969,19 +1966,19 @@
         <v>11</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="C77" s="2">
         <v>25216406</v>
       </c>
       <c r="D77" s="2">
-        <v>48.89</v>
+        <v>5</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -1989,13 +1986,13 @@
         <v>11</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C78" s="2">
         <v>25216406</v>
       </c>
-      <c r="D78" s="2">
-        <v>5</v>
+      <c r="D78" s="5">
+        <v>4.97</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>4</v>
@@ -2006,16 +2003,16 @@
     </row>
     <row r="79" spans="1:6">
       <c r="A79" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>132</v>
+        <v>85</v>
       </c>
       <c r="C79" s="2">
         <v>25216406</v>
       </c>
       <c r="D79" s="5">
-        <v>4.97</v>
+        <v>29045.65</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>4</v>
@@ -2029,39 +2026,39 @@
         <v>12</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>86</v>
+        <v>132</v>
       </c>
       <c r="C80" s="2">
         <v>25216406</v>
       </c>
       <c r="D80" s="5">
-        <v>29045.65</v>
+        <v>5.37</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>4</v>
+        <v>133</v>
       </c>
     </row>
     <row r="81" spans="1:6">
       <c r="A81" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>133</v>
+        <v>52</v>
       </c>
       <c r="C81" s="2">
         <v>25216406</v>
       </c>
-      <c r="D81" s="5">
-        <v>5.37</v>
+      <c r="D81" s="2">
+        <v>386057650000</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>134</v>
+        <v>53</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -2069,19 +2066,19 @@
         <v>14</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>53</v>
+        <v>83</v>
       </c>
       <c r="C82" s="2">
         <v>25216406</v>
       </c>
       <c r="D82" s="2">
-        <v>386057650000</v>
+        <v>15584515835.59</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>54</v>
+        <v>84</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -2089,39 +2086,39 @@
         <v>14</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="C83" s="2">
         <v>25216406</v>
       </c>
       <c r="D83" s="2">
-        <v>15584515835.59</v>
+        <v>632939341638</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>85</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84" spans="1:6">
       <c r="A84" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C84" s="2">
-        <v>25216406</v>
-      </c>
-      <c r="D84" s="2">
-        <v>632939341638</v>
+      <c r="C84" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -2129,19 +2126,19 @@
         <v>11</v>
       </c>
       <c r="B85" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D85" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E85" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C85" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E85" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="F85" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -2149,19 +2146,19 @@
         <v>11</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D86" s="6" t="s">
+      <c r="D86" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -2169,7 +2166,7 @@
         <v>11</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>4</v>
@@ -2178,30 +2175,30 @@
         <v>4</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D88" s="5" t="s">
-        <v>4</v>
+        <v>54</v>
+      </c>
+      <c r="C88" s="2">
+        <v>83191458</v>
+      </c>
+      <c r="D88" s="2">
+        <v>234162952118135</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -2209,19 +2206,19 @@
         <v>15</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C89" s="2">
         <v>83191458</v>
       </c>
       <c r="D89" s="2">
-        <v>234162952118135</v>
+        <v>271360000000</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>56</v>
+        <v>4</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -2229,39 +2226,39 @@
         <v>15</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="C90" s="2">
         <v>83191458</v>
       </c>
       <c r="D90" s="2">
-        <v>271360000000</v>
+        <v>366289414380.31</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>4</v>
+        <v>87</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C91" s="2">
-        <v>83191458</v>
-      </c>
-      <c r="D91" s="2">
-        <v>366289414380.31</v>
+        <v>423406343</v>
+      </c>
+      <c r="D91" s="5">
+        <v>5570.97</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>88</v>
+        <v>4</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -2274,8 +2271,8 @@
       <c r="C92" s="2">
         <v>423406343</v>
       </c>
-      <c r="D92" s="5">
-        <v>5570.97</v>
+      <c r="D92" s="2">
+        <v>2421.7600000000002</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>4</v>
@@ -2295,7 +2292,7 @@
         <v>423406343</v>
       </c>
       <c r="D93" s="2">
-        <v>2421.7600000000002</v>
+        <v>412796.66</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>4</v>
@@ -2306,16 +2303,16 @@
     </row>
     <row r="94" spans="1:6">
       <c r="A94" s="2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="C94" s="2">
-        <v>423406343</v>
+        <v>25216406</v>
       </c>
       <c r="D94" s="2">
-        <v>412796.66</v>
+        <v>473420.2</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>4</v>
@@ -2326,182 +2323,182 @@
     </row>
     <row r="95" spans="1:6">
       <c r="A95" s="2" t="s">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="C95" s="2">
-        <v>25216406</v>
+        <v>101527929</v>
       </c>
       <c r="D95" s="2">
-        <v>473420.2</v>
+        <v>778263.9</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>4</v>
+        <v>124</v>
       </c>
     </row>
     <row r="96" spans="1:6">
       <c r="A96" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C96" s="2">
         <v>101527929</v>
       </c>
-      <c r="D96" s="2">
-        <v>778263.9</v>
+      <c r="D96" s="5">
+        <v>209000</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>125</v>
+        <v>4</v>
       </c>
     </row>
     <row r="97" spans="1:6">
       <c r="A97" s="2" t="s">
-        <v>114</v>
+        <v>26</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>126</v>
+        <v>54</v>
       </c>
       <c r="C97" s="2">
-        <v>101527929</v>
-      </c>
-      <c r="D97" s="5">
-        <v>209000</v>
+        <v>83191458</v>
+      </c>
+      <c r="D97" s="2">
+        <v>39265232.859999999</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
     </row>
     <row r="98" spans="1:6">
       <c r="A98" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="C98" s="2">
-        <v>83191458</v>
-      </c>
-      <c r="D98" s="2">
-        <v>39265232.859999999</v>
+        <v>86837700</v>
+      </c>
+      <c r="D98" s="5">
+        <v>613304.94999999995</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>56</v>
+        <v>4</v>
       </c>
     </row>
     <row r="99" spans="1:6">
       <c r="A99" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="C99" s="2">
-        <v>86837700</v>
-      </c>
-      <c r="D99" s="5">
-        <v>613304.94999999995</v>
+        <v>83191458</v>
+      </c>
+      <c r="D99" s="2">
+        <v>17357276.120000001</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
     </row>
     <row r="100" spans="1:6">
       <c r="A100" s="2" t="s">
-        <v>30</v>
+        <v>92</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="C100" s="2">
-        <v>83191458</v>
+        <v>25216406</v>
       </c>
       <c r="D100" s="2">
-        <v>17357276.120000001</v>
+        <v>64333.279999999999</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>56</v>
+        <v>84</v>
       </c>
     </row>
     <row r="101" spans="1:6">
       <c r="A101" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B101" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="B101" s="2" t="s">
-        <v>84</v>
       </c>
       <c r="C101" s="2">
         <v>25216406</v>
       </c>
       <c r="D101" s="2">
-        <v>64333.279999999999</v>
+        <v>1045412.19</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="102" spans="1:6">
       <c r="A102" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="C102" s="2">
         <v>25216406</v>
       </c>
       <c r="D102" s="2">
-        <v>1045412.19</v>
+        <v>2500001</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
     </row>
     <row r="103" spans="1:6">
       <c r="A103" s="2" t="s">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C103" s="2">
-        <v>25216406</v>
-      </c>
-      <c r="D103" s="2">
-        <v>2500001</v>
+      <c r="C103" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -2509,19 +2506,19 @@
         <v>11</v>
       </c>
       <c r="B104" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E104" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C104" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E104" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="F104" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -2529,7 +2526,7 @@
         <v>11</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C105" s="2" t="s">
         <v>4</v>
@@ -2538,10 +2535,10 @@
         <v>4</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -2549,7 +2546,7 @@
         <v>11</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C106" s="2" t="s">
         <v>4</v>
@@ -2558,30 +2555,30 @@
         <v>4</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" s="2" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>4</v>
+        <v>56</v>
+      </c>
+      <c r="C107" s="2">
+        <v>83191458</v>
+      </c>
+      <c r="D107" s="2">
+        <v>2500000</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>76</v>
+        <v>4</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>83</v>
+        <v>4</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -2589,19 +2586,19 @@
         <v>29</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C108" s="2">
-        <v>83191458</v>
-      </c>
-      <c r="D108" s="2">
-        <v>2500000</v>
+        <v>95</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>4</v>
+        <v>96</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -2609,19 +2606,19 @@
         <v>29</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C109" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D109" s="5" t="s">
+      <c r="D109" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -2629,7 +2626,7 @@
         <v>29</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C110" s="2" t="s">
         <v>4</v>
@@ -2638,10 +2635,10 @@
         <v>4</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -2649,53 +2646,53 @@
         <v>29</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C111" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D111" s="2" t="s">
-        <v>4</v>
+        <v>86</v>
+      </c>
+      <c r="C111" s="2">
+        <v>83191458</v>
+      </c>
+      <c r="D111" s="2">
+        <v>26954</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
     </row>
     <row r="112" spans="1:6">
       <c r="A112" s="2" t="s">
-        <v>29</v>
+        <v>134</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="C112" s="2">
-        <v>83191458</v>
-      </c>
-      <c r="D112" s="2">
-        <v>26954</v>
+        <v>25216406</v>
+      </c>
+      <c r="D112" s="3">
+        <v>14303345.08</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>88</v>
+        <v>4</v>
       </c>
     </row>
     <row r="113" spans="1:6">
       <c r="A113" s="2" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>74</v>
+        <v>125</v>
       </c>
       <c r="C113" s="2">
-        <v>25216406</v>
+        <v>101527929</v>
       </c>
       <c r="D113" s="3">
-        <v>14303345.08</v>
+        <v>4015169.7</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>4</v>
@@ -2706,56 +2703,56 @@
     </row>
     <row r="114" spans="1:6">
       <c r="A114" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C114" s="2">
         <v>101527929</v>
       </c>
       <c r="D114" s="3">
-        <v>4015169.7</v>
+        <v>6168237.7300000004</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>4</v>
+        <v>124</v>
       </c>
     </row>
     <row r="115" spans="1:6">
       <c r="A115" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>124</v>
+        <v>56</v>
       </c>
       <c r="C115" s="2">
-        <v>101527929</v>
+        <v>83191458</v>
       </c>
       <c r="D115" s="3">
-        <v>6168237.7300000004</v>
+        <v>20469173.030000001</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>125</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116" spans="1:6">
       <c r="A116" s="2" t="s">
-        <v>115</v>
+        <v>24</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>57</v>
+        <v>125</v>
       </c>
       <c r="C116" s="2">
-        <v>83191458</v>
+        <v>101527929</v>
       </c>
       <c r="D116" s="3">
-        <v>20469173.030000001</v>
+        <v>412000</v>
       </c>
       <c r="E116" s="2" t="s">
         <v>4</v>
@@ -2766,16 +2763,16 @@
     </row>
     <row r="117" spans="1:6">
       <c r="A117" s="2" t="s">
-        <v>24</v>
+        <v>117</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>126</v>
+        <v>73</v>
       </c>
       <c r="C117" s="2">
-        <v>101527929</v>
+        <v>25216406</v>
       </c>
       <c r="D117" s="3">
-        <v>412000</v>
+        <v>537679.1</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>4</v>
@@ -2786,22 +2783,22 @@
     </row>
     <row r="118" spans="1:6">
       <c r="A118" s="2" t="s">
-        <v>118</v>
+        <v>11</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C118" s="2">
-        <v>25216406</v>
-      </c>
-      <c r="D118" s="3">
-        <v>537679.1</v>
+      <c r="C118" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>4</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
     </row>
     <row r="119" spans="1:6">
@@ -2809,19 +2806,19 @@
         <v>11</v>
       </c>
       <c r="B119" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E119" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C119" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D119" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="F119" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="120" spans="1:6">
@@ -2829,7 +2826,7 @@
         <v>11</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C120" s="2" t="s">
         <v>4</v>
@@ -2838,10 +2835,10 @@
         <v>4</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="121" spans="1:6">
@@ -2849,7 +2846,7 @@
         <v>11</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C121" s="2" t="s">
         <v>4</v>
@@ -2858,30 +2855,30 @@
         <v>4</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="122" spans="1:6">
       <c r="A122" s="2" t="s">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C122" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D122" s="3" t="s">
-        <v>4</v>
+        <v>52</v>
+      </c>
+      <c r="C122" s="2">
+        <v>25216406</v>
+      </c>
+      <c r="D122" s="3">
+        <v>44805205.200000003</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>83</v>
+        <v>53</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -2889,19 +2886,19 @@
         <v>120</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C123" s="2">
-        <v>25216406</v>
+        <v>83191458</v>
       </c>
       <c r="D123" s="3">
-        <v>44805205.200000003</v>
+        <v>297692</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -2909,39 +2906,39 @@
         <v>121</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C124" s="2">
         <v>83191458</v>
       </c>
       <c r="D124" s="3">
-        <v>297692</v>
+        <v>76466743.670000002</v>
       </c>
       <c r="E124" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="125" spans="1:6">
       <c r="A125" s="2" t="s">
-        <v>122</v>
+        <v>35</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>55</v>
+        <v>101</v>
       </c>
       <c r="C125" s="2">
-        <v>83191458</v>
+        <v>104607823</v>
       </c>
       <c r="D125" s="3">
-        <v>76466743.670000002</v>
+        <v>27987852.739999998</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>56</v>
+        <v>4</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -2955,7 +2952,7 @@
         <v>104607823</v>
       </c>
       <c r="D126" s="3">
-        <v>27987852.739999998</v>
+        <v>766000.99</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>4</v>
@@ -2966,16 +2963,16 @@
     </row>
     <row r="127" spans="1:6">
       <c r="A127" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="C127" s="2">
-        <v>104607823</v>
+        <v>25216406</v>
       </c>
       <c r="D127" s="3">
-        <v>766000.99</v>
+        <v>10000000</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>4</v>
@@ -2989,19 +2986,19 @@
         <v>33</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>74</v>
+        <v>52</v>
       </c>
       <c r="C128" s="2">
         <v>25216406</v>
       </c>
       <c r="D128" s="3">
-        <v>10000000</v>
+        <v>15156000.02</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>4</v>
+        <v>53</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -3009,39 +3006,39 @@
         <v>33</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>53</v>
+        <v>83</v>
       </c>
       <c r="C129" s="2">
         <v>25216406</v>
       </c>
       <c r="D129" s="3">
-        <v>15156000.02</v>
+        <v>684193.22</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>54</v>
+        <v>84</v>
       </c>
     </row>
     <row r="130" spans="1:6">
       <c r="A130" s="2" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>84</v>
+        <v>135</v>
       </c>
       <c r="C130" s="2">
-        <v>25216406</v>
+        <v>6229557</v>
       </c>
       <c r="D130" s="3">
-        <v>684193.22</v>
+        <v>268855.80028187</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>85</v>
+        <v>4</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -3049,13 +3046,13 @@
         <v>9</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="C131" s="2">
         <v>6229557</v>
       </c>
       <c r="D131" s="3">
-        <v>268855.80028187</v>
+        <v>187180.2115</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>4</v>
@@ -3069,13 +3066,13 @@
         <v>9</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="C132" s="2">
         <v>6229557</v>
       </c>
       <c r="D132" s="3">
-        <v>187180.2115</v>
+        <v>156897.95726011001</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>4</v>
@@ -3089,13 +3086,13 @@
         <v>9</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>137</v>
+        <v>103</v>
       </c>
       <c r="C133" s="2">
         <v>6229557</v>
       </c>
       <c r="D133" s="3">
-        <v>156897.95726011001</v>
+        <v>369891003.48900002</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>4</v>
@@ -3105,7 +3102,7 @@
       </c>
     </row>
     <row r="134" spans="1:6">
-      <c r="A134" s="2" t="s">
+      <c r="A134" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B134" s="2" t="s">
@@ -3115,7 +3112,7 @@
         <v>6229557</v>
       </c>
       <c r="D134" s="3">
-        <v>369891003.48900002</v>
+        <v>66066923.393727899</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>4</v>
@@ -3125,7 +3122,7 @@
       </c>
     </row>
     <row r="135" spans="1:6">
-      <c r="A135" s="8" t="s">
+      <c r="A135" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B135" s="2" t="s">
@@ -3135,7 +3132,7 @@
         <v>6229557</v>
       </c>
       <c r="D135" s="3">
-        <v>66066923.393727899</v>
+        <v>2866993.9984026002</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>4</v>
@@ -3155,7 +3152,7 @@
         <v>6229557</v>
       </c>
       <c r="D136" s="3">
-        <v>2866993.9984026002</v>
+        <v>2647816.5263509499</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>4</v>
@@ -3175,7 +3172,7 @@
         <v>6229557</v>
       </c>
       <c r="D137" s="3">
-        <v>2647816.5263509499</v>
+        <v>1457329.6256335201</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>4</v>
@@ -3195,7 +3192,7 @@
         <v>6229557</v>
       </c>
       <c r="D138" s="3">
-        <v>1457329.6256335201</v>
+        <v>1066964.2965422401</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>4</v>
@@ -3215,7 +3212,7 @@
         <v>6229557</v>
       </c>
       <c r="D139" s="3">
-        <v>1066964.2965422401</v>
+        <v>850746.71291593998</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>4</v>
@@ -3235,7 +3232,7 @@
         <v>6229557</v>
       </c>
       <c r="D140" s="3">
-        <v>850746.71291593998</v>
+        <v>579364.12614367995</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>4</v>
@@ -3255,7 +3252,7 @@
         <v>6229557</v>
       </c>
       <c r="D141" s="3">
-        <v>579364.12614367995</v>
+        <v>538350.47626451997</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>4</v>
@@ -3275,7 +3272,7 @@
         <v>6229557</v>
       </c>
       <c r="D142" s="3">
-        <v>538350.47626451997</v>
+        <v>127419.4406821</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>4</v>
@@ -3289,13 +3286,13 @@
         <v>9</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="C143" s="2">
         <v>6229557</v>
       </c>
       <c r="D143" s="3">
-        <v>127419.4406821</v>
+        <v>104766.0303</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>4</v>
@@ -3315,7 +3312,7 @@
         <v>6229557</v>
       </c>
       <c r="D144" s="3">
-        <v>104766.0303</v>
+        <v>4535998.9539999999</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>4</v>
@@ -3335,7 +3332,7 @@
         <v>6229557</v>
       </c>
       <c r="D145" s="3">
-        <v>4535998.9539999999</v>
+        <v>1054996.6370000001</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>4</v>
@@ -3354,8 +3351,8 @@
       <c r="C146" s="2">
         <v>6229557</v>
       </c>
-      <c r="D146" s="3">
-        <v>1054996.6370000001</v>
+      <c r="D146" s="2">
+        <v>1018930.2</v>
       </c>
       <c r="E146" s="2" t="s">
         <v>4</v>
@@ -3375,7 +3372,7 @@
         <v>6229557</v>
       </c>
       <c r="D147" s="2">
-        <v>1018930.2</v>
+        <v>497999.43900000001</v>
       </c>
       <c r="E147" s="2" t="s">
         <v>4</v>
@@ -3395,32 +3392,12 @@
         <v>6229557</v>
       </c>
       <c r="D148" s="2">
-        <v>497999.43900000001</v>
+        <v>244998.32</v>
       </c>
       <c r="E148" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="149" spans="1:6">
-      <c r="A149" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C149" s="2">
-        <v>6229557</v>
-      </c>
-      <c r="D149" s="2">
-        <v>244998.32</v>
-      </c>
-      <c r="E149" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F149" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>